<commit_message>
feat: add flashlight toggle functionality and update UI elements in index.html; update session ID in config.json; replace backup Excel files
</commit_message>
<xml_diff>
--- a/py_test_ui/EXCEL FILE/backuprecordCal_PM.xlsx
+++ b/py_test_ui/EXCEL FILE/backuprecordCal_PM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\forms-1\py_test_ui\EXCEL FILE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB81E2BB-AA3F-4A3B-98AD-519662839D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_50ED3F369565C60E62355476585DCE3A874AAE20" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12304" uniqueCount="1282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13314" uniqueCount="1395">
   <si>
     <t>N0</t>
   </si>
@@ -3866,6 +3866,345 @@
   </si>
   <si>
     <t>PYT3_09985</t>
+  </si>
+  <si>
+    <t>33843</t>
+  </si>
+  <si>
+    <t>PYT3_00852</t>
+  </si>
+  <si>
+    <t>25/06/2026</t>
+  </si>
+  <si>
+    <t>405069</t>
+  </si>
+  <si>
+    <t>PYT3_09317</t>
+  </si>
+  <si>
+    <t>405070</t>
+  </si>
+  <si>
+    <t>PYT3_09318</t>
+  </si>
+  <si>
+    <t>32212</t>
+  </si>
+  <si>
+    <t>PYT3_00303</t>
+  </si>
+  <si>
+    <t>32220</t>
+  </si>
+  <si>
+    <t>PYT3_00311</t>
+  </si>
+  <si>
+    <t>39095</t>
+  </si>
+  <si>
+    <t>PYT3_02472</t>
+  </si>
+  <si>
+    <t>40220</t>
+  </si>
+  <si>
+    <t>PYT3_02627</t>
+  </si>
+  <si>
+    <t>110113</t>
+  </si>
+  <si>
+    <t>PYT3_04832</t>
+  </si>
+  <si>
+    <t>261025</t>
+  </si>
+  <si>
+    <t>PYT3_07170</t>
+  </si>
+  <si>
+    <t>376333</t>
+  </si>
+  <si>
+    <t>PYT3_09010</t>
+  </si>
+  <si>
+    <t>252387</t>
+  </si>
+  <si>
+    <t>PYT3_06942</t>
+  </si>
+  <si>
+    <t>259344</t>
+  </si>
+  <si>
+    <t>PYT3_07046</t>
+  </si>
+  <si>
+    <t>259345</t>
+  </si>
+  <si>
+    <t>PYT3_07047</t>
+  </si>
+  <si>
+    <t>259347</t>
+  </si>
+  <si>
+    <t>PYT3_07049</t>
+  </si>
+  <si>
+    <t>260558</t>
+  </si>
+  <si>
+    <t>PYT3_07075</t>
+  </si>
+  <si>
+    <t>314152</t>
+  </si>
+  <si>
+    <t>PYT3_08213</t>
+  </si>
+  <si>
+    <t>408388</t>
+  </si>
+  <si>
+    <t>PYT3_09498</t>
+  </si>
+  <si>
+    <t>408389</t>
+  </si>
+  <si>
+    <t>PYT3_09499</t>
+  </si>
+  <si>
+    <t>411762</t>
+  </si>
+  <si>
+    <t>PYT3_09545</t>
+  </si>
+  <si>
+    <t>411763</t>
+  </si>
+  <si>
+    <t>PYT3_09546</t>
+  </si>
+  <si>
+    <t>412772</t>
+  </si>
+  <si>
+    <t>PYT3_09595</t>
+  </si>
+  <si>
+    <t>412806</t>
+  </si>
+  <si>
+    <t>PYT3_09596</t>
+  </si>
+  <si>
+    <t>36490</t>
+  </si>
+  <si>
+    <t>PYT3_01160</t>
+  </si>
+  <si>
+    <t>33863</t>
+  </si>
+  <si>
+    <t>PYT3_00872</t>
+  </si>
+  <si>
+    <t>36541</t>
+  </si>
+  <si>
+    <t>PYT3_01211</t>
+  </si>
+  <si>
+    <t>37956</t>
+  </si>
+  <si>
+    <t>PYT3_01730</t>
+  </si>
+  <si>
+    <t>328195</t>
+  </si>
+  <si>
+    <t>PYT3_08488</t>
+  </si>
+  <si>
+    <t>308882</t>
+  </si>
+  <si>
+    <t>PYT3_08117</t>
+  </si>
+  <si>
+    <t>380475</t>
+  </si>
+  <si>
+    <t>PYT3_09075</t>
+  </si>
+  <si>
+    <t>398937</t>
+  </si>
+  <si>
+    <t>PYT3_09232</t>
+  </si>
+  <si>
+    <t>398938</t>
+  </si>
+  <si>
+    <t>PYT3_09233</t>
+  </si>
+  <si>
+    <t>40104</t>
+  </si>
+  <si>
+    <t>PYT3_02511</t>
+  </si>
+  <si>
+    <t>109948</t>
+  </si>
+  <si>
+    <t>PYT3_04668</t>
+  </si>
+  <si>
+    <t>401704</t>
+  </si>
+  <si>
+    <t>PYT3_09294</t>
+  </si>
+  <si>
+    <t>397604</t>
+  </si>
+  <si>
+    <t>PYT3_09200</t>
+  </si>
+  <si>
+    <t>40505</t>
+  </si>
+  <si>
+    <t>PYT3_02902</t>
+  </si>
+  <si>
+    <t>109998</t>
+  </si>
+  <si>
+    <t>PYT3_04718</t>
+  </si>
+  <si>
+    <t>109999</t>
+  </si>
+  <si>
+    <t>PYT3_04719</t>
+  </si>
+  <si>
+    <t>110000</t>
+  </si>
+  <si>
+    <t>PYT3_04720</t>
+  </si>
+  <si>
+    <t>110002</t>
+  </si>
+  <si>
+    <t>PYT3_04722</t>
+  </si>
+  <si>
+    <t>110011</t>
+  </si>
+  <si>
+    <t>PYT3_04731</t>
+  </si>
+  <si>
+    <t>425930</t>
+  </si>
+  <si>
+    <t>PYT3_09944</t>
+  </si>
+  <si>
+    <t>38816</t>
+  </si>
+  <si>
+    <t>PYT3_02288</t>
+  </si>
+  <si>
+    <t>38823</t>
+  </si>
+  <si>
+    <t>PYT3_02295</t>
+  </si>
+  <si>
+    <t>40138</t>
+  </si>
+  <si>
+    <t>PYT3_02545</t>
+  </si>
+  <si>
+    <t>375695</t>
+  </si>
+  <si>
+    <t>PYT3_08994</t>
+  </si>
+  <si>
+    <t>379742</t>
+  </si>
+  <si>
+    <t>PYT3_09064</t>
+  </si>
+  <si>
+    <t>425939</t>
+  </si>
+  <si>
+    <t>PYT3_09953</t>
+  </si>
+  <si>
+    <t>36481</t>
+  </si>
+  <si>
+    <t>PYT3_01151</t>
+  </si>
+  <si>
+    <t>40143</t>
+  </si>
+  <si>
+    <t>PYT3_02550</t>
+  </si>
+  <si>
+    <t>179410</t>
+  </si>
+  <si>
+    <t>PYT3_05853</t>
+  </si>
+  <si>
+    <t>216627</t>
+  </si>
+  <si>
+    <t>PYT3_06552</t>
+  </si>
+  <si>
+    <t>260617</t>
+  </si>
+  <si>
+    <t>PYT3_07102</t>
+  </si>
+  <si>
+    <t>323433</t>
+  </si>
+  <si>
+    <t>PYT3_08376</t>
+  </si>
+  <si>
+    <t>40170</t>
+  </si>
+  <si>
+    <t>PYT3D_02577</t>
+  </si>
+  <si>
+    <t>40177</t>
+  </si>
+  <si>
+    <t>PYT3D_02584</t>
   </si>
 </sst>
 </file>
@@ -4229,7 +4568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z615"/>
+  <dimension ref="A1:Z671"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
@@ -9761,6 +10100,12 @@
       <c r="S89" t="s">
         <v>39</v>
       </c>
+      <c r="V89" t="s">
+        <v>40</v>
+      </c>
+      <c r="W89" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="90" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B90" t="s">
@@ -42372,6 +42717,3142 @@
       </c>
       <c r="W615" t="s">
         <v>40</v>
+      </c>
+    </row>
+    <row r="616" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B616" t="s">
+        <v>1282</v>
+      </c>
+      <c r="C616" t="s">
+        <v>1283</v>
+      </c>
+      <c r="D616" t="s">
+        <v>28</v>
+      </c>
+      <c r="E616" t="s">
+        <v>29</v>
+      </c>
+      <c r="F616" t="s">
+        <v>30</v>
+      </c>
+      <c r="G616" t="s">
+        <v>31</v>
+      </c>
+      <c r="H616" t="s">
+        <v>32</v>
+      </c>
+      <c r="I616" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J616" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K616" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L616" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M616" t="s">
+        <v>34</v>
+      </c>
+      <c r="N616" t="s">
+        <v>35</v>
+      </c>
+      <c r="O616" t="s">
+        <v>36</v>
+      </c>
+      <c r="P616" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q616" t="s">
+        <v>38</v>
+      </c>
+      <c r="R616" t="s">
+        <v>38</v>
+      </c>
+      <c r="S616" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="617" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B617" t="s">
+        <v>1285</v>
+      </c>
+      <c r="C617" t="s">
+        <v>1286</v>
+      </c>
+      <c r="D617" t="s">
+        <v>28</v>
+      </c>
+      <c r="E617" t="s">
+        <v>29</v>
+      </c>
+      <c r="F617" t="s">
+        <v>30</v>
+      </c>
+      <c r="G617" t="s">
+        <v>31</v>
+      </c>
+      <c r="H617" t="s">
+        <v>32</v>
+      </c>
+      <c r="I617" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J617" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K617" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L617" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M617" t="s">
+        <v>34</v>
+      </c>
+      <c r="N617" t="s">
+        <v>35</v>
+      </c>
+      <c r="O617" t="s">
+        <v>36</v>
+      </c>
+      <c r="P617" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q617" t="s">
+        <v>38</v>
+      </c>
+      <c r="R617" t="s">
+        <v>38</v>
+      </c>
+      <c r="S617" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="618" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B618" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C618" t="s">
+        <v>1288</v>
+      </c>
+      <c r="D618" t="s">
+        <v>28</v>
+      </c>
+      <c r="E618" t="s">
+        <v>29</v>
+      </c>
+      <c r="F618" t="s">
+        <v>30</v>
+      </c>
+      <c r="G618" t="s">
+        <v>31</v>
+      </c>
+      <c r="H618" t="s">
+        <v>32</v>
+      </c>
+      <c r="I618" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J618" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K618" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L618" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M618" t="s">
+        <v>34</v>
+      </c>
+      <c r="N618" t="s">
+        <v>35</v>
+      </c>
+      <c r="O618" t="s">
+        <v>36</v>
+      </c>
+      <c r="P618" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q618" t="s">
+        <v>38</v>
+      </c>
+      <c r="R618" t="s">
+        <v>38</v>
+      </c>
+      <c r="S618" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="619" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B619" t="s">
+        <v>1289</v>
+      </c>
+      <c r="C619" t="s">
+        <v>1290</v>
+      </c>
+      <c r="D619" t="s">
+        <v>28</v>
+      </c>
+      <c r="E619" t="s">
+        <v>29</v>
+      </c>
+      <c r="F619" t="s">
+        <v>30</v>
+      </c>
+      <c r="G619" t="s">
+        <v>31</v>
+      </c>
+      <c r="H619" t="s">
+        <v>32</v>
+      </c>
+      <c r="I619" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J619" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K619" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L619" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M619" t="s">
+        <v>34</v>
+      </c>
+      <c r="N619" t="s">
+        <v>35</v>
+      </c>
+      <c r="O619" t="s">
+        <v>36</v>
+      </c>
+      <c r="P619" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q619" t="s">
+        <v>38</v>
+      </c>
+      <c r="R619" t="s">
+        <v>38</v>
+      </c>
+      <c r="S619" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="620" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B620" t="s">
+        <v>1291</v>
+      </c>
+      <c r="C620" t="s">
+        <v>1292</v>
+      </c>
+      <c r="D620" t="s">
+        <v>28</v>
+      </c>
+      <c r="E620" t="s">
+        <v>29</v>
+      </c>
+      <c r="F620" t="s">
+        <v>30</v>
+      </c>
+      <c r="G620" t="s">
+        <v>31</v>
+      </c>
+      <c r="H620" t="s">
+        <v>32</v>
+      </c>
+      <c r="I620" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J620" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K620" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L620" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M620" t="s">
+        <v>34</v>
+      </c>
+      <c r="N620" t="s">
+        <v>35</v>
+      </c>
+      <c r="O620" t="s">
+        <v>36</v>
+      </c>
+      <c r="P620" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q620" t="s">
+        <v>38</v>
+      </c>
+      <c r="R620" t="s">
+        <v>38</v>
+      </c>
+      <c r="S620" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="621" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B621" t="s">
+        <v>1293</v>
+      </c>
+      <c r="C621" t="s">
+        <v>1294</v>
+      </c>
+      <c r="D621" t="s">
+        <v>28</v>
+      </c>
+      <c r="E621" t="s">
+        <v>29</v>
+      </c>
+      <c r="F621" t="s">
+        <v>30</v>
+      </c>
+      <c r="G621" t="s">
+        <v>31</v>
+      </c>
+      <c r="H621" t="s">
+        <v>32</v>
+      </c>
+      <c r="I621" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J621" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K621" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L621" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M621" t="s">
+        <v>34</v>
+      </c>
+      <c r="N621" t="s">
+        <v>35</v>
+      </c>
+      <c r="O621" t="s">
+        <v>36</v>
+      </c>
+      <c r="P621" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q621" t="s">
+        <v>38</v>
+      </c>
+      <c r="R621" t="s">
+        <v>38</v>
+      </c>
+      <c r="S621" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="622" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B622" t="s">
+        <v>1295</v>
+      </c>
+      <c r="C622" t="s">
+        <v>1296</v>
+      </c>
+      <c r="D622" t="s">
+        <v>28</v>
+      </c>
+      <c r="E622" t="s">
+        <v>29</v>
+      </c>
+      <c r="F622" t="s">
+        <v>30</v>
+      </c>
+      <c r="G622" t="s">
+        <v>31</v>
+      </c>
+      <c r="H622" t="s">
+        <v>32</v>
+      </c>
+      <c r="I622" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J622" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K622" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L622" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M622" t="s">
+        <v>34</v>
+      </c>
+      <c r="N622" t="s">
+        <v>35</v>
+      </c>
+      <c r="O622" t="s">
+        <v>36</v>
+      </c>
+      <c r="P622" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q622" t="s">
+        <v>38</v>
+      </c>
+      <c r="R622" t="s">
+        <v>38</v>
+      </c>
+      <c r="S622" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="623" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B623" t="s">
+        <v>1297</v>
+      </c>
+      <c r="C623" t="s">
+        <v>1298</v>
+      </c>
+      <c r="D623" t="s">
+        <v>28</v>
+      </c>
+      <c r="E623" t="s">
+        <v>29</v>
+      </c>
+      <c r="F623" t="s">
+        <v>30</v>
+      </c>
+      <c r="G623" t="s">
+        <v>31</v>
+      </c>
+      <c r="H623" t="s">
+        <v>32</v>
+      </c>
+      <c r="I623" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J623" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K623" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L623" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M623" t="s">
+        <v>34</v>
+      </c>
+      <c r="N623" t="s">
+        <v>35</v>
+      </c>
+      <c r="O623" t="s">
+        <v>36</v>
+      </c>
+      <c r="P623" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q623" t="s">
+        <v>38</v>
+      </c>
+      <c r="R623" t="s">
+        <v>38</v>
+      </c>
+      <c r="S623" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="624" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B624" t="s">
+        <v>1299</v>
+      </c>
+      <c r="C624" t="s">
+        <v>1300</v>
+      </c>
+      <c r="D624" t="s">
+        <v>28</v>
+      </c>
+      <c r="E624" t="s">
+        <v>29</v>
+      </c>
+      <c r="F624" t="s">
+        <v>30</v>
+      </c>
+      <c r="G624" t="s">
+        <v>31</v>
+      </c>
+      <c r="H624" t="s">
+        <v>32</v>
+      </c>
+      <c r="I624" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J624" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K624" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L624" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M624" t="s">
+        <v>34</v>
+      </c>
+      <c r="N624" t="s">
+        <v>35</v>
+      </c>
+      <c r="O624" t="s">
+        <v>36</v>
+      </c>
+      <c r="P624" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q624" t="s">
+        <v>38</v>
+      </c>
+      <c r="R624" t="s">
+        <v>38</v>
+      </c>
+      <c r="S624" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="625" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B625" t="s">
+        <v>1301</v>
+      </c>
+      <c r="C625" t="s">
+        <v>1302</v>
+      </c>
+      <c r="D625" t="s">
+        <v>28</v>
+      </c>
+      <c r="E625" t="s">
+        <v>29</v>
+      </c>
+      <c r="F625" t="s">
+        <v>30</v>
+      </c>
+      <c r="G625" t="s">
+        <v>31</v>
+      </c>
+      <c r="H625" t="s">
+        <v>32</v>
+      </c>
+      <c r="I625" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J625" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K625" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L625" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M625" t="s">
+        <v>34</v>
+      </c>
+      <c r="N625" t="s">
+        <v>35</v>
+      </c>
+      <c r="O625" t="s">
+        <v>36</v>
+      </c>
+      <c r="P625" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q625" t="s">
+        <v>38</v>
+      </c>
+      <c r="R625" t="s">
+        <v>38</v>
+      </c>
+      <c r="S625" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="626" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B626" t="s">
+        <v>1303</v>
+      </c>
+      <c r="C626" t="s">
+        <v>1304</v>
+      </c>
+      <c r="D626" t="s">
+        <v>28</v>
+      </c>
+      <c r="E626" t="s">
+        <v>29</v>
+      </c>
+      <c r="F626" t="s">
+        <v>30</v>
+      </c>
+      <c r="G626" t="s">
+        <v>31</v>
+      </c>
+      <c r="H626" t="s">
+        <v>32</v>
+      </c>
+      <c r="I626" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J626" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K626" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L626" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M626" t="s">
+        <v>34</v>
+      </c>
+      <c r="N626" t="s">
+        <v>35</v>
+      </c>
+      <c r="O626" t="s">
+        <v>36</v>
+      </c>
+      <c r="P626" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q626" t="s">
+        <v>38</v>
+      </c>
+      <c r="R626" t="s">
+        <v>38</v>
+      </c>
+      <c r="S626" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="627" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B627" t="s">
+        <v>1305</v>
+      </c>
+      <c r="C627" t="s">
+        <v>1306</v>
+      </c>
+      <c r="D627" t="s">
+        <v>28</v>
+      </c>
+      <c r="E627" t="s">
+        <v>29</v>
+      </c>
+      <c r="F627" t="s">
+        <v>30</v>
+      </c>
+      <c r="G627" t="s">
+        <v>31</v>
+      </c>
+      <c r="H627" t="s">
+        <v>32</v>
+      </c>
+      <c r="I627" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J627" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K627" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L627" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M627" t="s">
+        <v>34</v>
+      </c>
+      <c r="N627" t="s">
+        <v>35</v>
+      </c>
+      <c r="O627" t="s">
+        <v>36</v>
+      </c>
+      <c r="P627" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q627" t="s">
+        <v>38</v>
+      </c>
+      <c r="R627" t="s">
+        <v>38</v>
+      </c>
+      <c r="S627" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="628" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B628" t="s">
+        <v>1307</v>
+      </c>
+      <c r="C628" t="s">
+        <v>1308</v>
+      </c>
+      <c r="D628" t="s">
+        <v>28</v>
+      </c>
+      <c r="E628" t="s">
+        <v>29</v>
+      </c>
+      <c r="F628" t="s">
+        <v>30</v>
+      </c>
+      <c r="G628" t="s">
+        <v>31</v>
+      </c>
+      <c r="H628" t="s">
+        <v>32</v>
+      </c>
+      <c r="I628" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J628" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K628" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L628" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M628" t="s">
+        <v>34</v>
+      </c>
+      <c r="N628" t="s">
+        <v>35</v>
+      </c>
+      <c r="O628" t="s">
+        <v>36</v>
+      </c>
+      <c r="P628" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q628" t="s">
+        <v>38</v>
+      </c>
+      <c r="R628" t="s">
+        <v>38</v>
+      </c>
+      <c r="S628" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="629" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B629" t="s">
+        <v>1309</v>
+      </c>
+      <c r="C629" t="s">
+        <v>1310</v>
+      </c>
+      <c r="D629" t="s">
+        <v>28</v>
+      </c>
+      <c r="E629" t="s">
+        <v>29</v>
+      </c>
+      <c r="F629" t="s">
+        <v>30</v>
+      </c>
+      <c r="G629" t="s">
+        <v>31</v>
+      </c>
+      <c r="H629" t="s">
+        <v>32</v>
+      </c>
+      <c r="I629" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J629" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K629" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L629" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M629" t="s">
+        <v>34</v>
+      </c>
+      <c r="N629" t="s">
+        <v>35</v>
+      </c>
+      <c r="O629" t="s">
+        <v>36</v>
+      </c>
+      <c r="P629" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q629" t="s">
+        <v>38</v>
+      </c>
+      <c r="R629" t="s">
+        <v>38</v>
+      </c>
+      <c r="S629" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="630" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B630" t="s">
+        <v>1311</v>
+      </c>
+      <c r="C630" t="s">
+        <v>1312</v>
+      </c>
+      <c r="D630" t="s">
+        <v>28</v>
+      </c>
+      <c r="E630" t="s">
+        <v>29</v>
+      </c>
+      <c r="F630" t="s">
+        <v>30</v>
+      </c>
+      <c r="G630" t="s">
+        <v>31</v>
+      </c>
+      <c r="H630" t="s">
+        <v>32</v>
+      </c>
+      <c r="I630" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J630" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K630" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L630" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M630" t="s">
+        <v>34</v>
+      </c>
+      <c r="N630" t="s">
+        <v>35</v>
+      </c>
+      <c r="O630" t="s">
+        <v>36</v>
+      </c>
+      <c r="P630" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q630" t="s">
+        <v>38</v>
+      </c>
+      <c r="R630" t="s">
+        <v>38</v>
+      </c>
+      <c r="S630" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="631" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B631" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C631" t="s">
+        <v>1314</v>
+      </c>
+      <c r="D631" t="s">
+        <v>28</v>
+      </c>
+      <c r="E631" t="s">
+        <v>29</v>
+      </c>
+      <c r="F631" t="s">
+        <v>30</v>
+      </c>
+      <c r="G631" t="s">
+        <v>31</v>
+      </c>
+      <c r="H631" t="s">
+        <v>32</v>
+      </c>
+      <c r="I631" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J631" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K631" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L631" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M631" t="s">
+        <v>34</v>
+      </c>
+      <c r="N631" t="s">
+        <v>35</v>
+      </c>
+      <c r="O631" t="s">
+        <v>36</v>
+      </c>
+      <c r="P631" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q631" t="s">
+        <v>38</v>
+      </c>
+      <c r="R631" t="s">
+        <v>38</v>
+      </c>
+      <c r="S631" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="632" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B632" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C632" t="s">
+        <v>1316</v>
+      </c>
+      <c r="D632" t="s">
+        <v>28</v>
+      </c>
+      <c r="E632" t="s">
+        <v>29</v>
+      </c>
+      <c r="F632" t="s">
+        <v>30</v>
+      </c>
+      <c r="G632" t="s">
+        <v>31</v>
+      </c>
+      <c r="H632" t="s">
+        <v>32</v>
+      </c>
+      <c r="I632" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J632" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K632" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L632" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M632" t="s">
+        <v>34</v>
+      </c>
+      <c r="N632" t="s">
+        <v>35</v>
+      </c>
+      <c r="O632" t="s">
+        <v>36</v>
+      </c>
+      <c r="P632" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q632" t="s">
+        <v>38</v>
+      </c>
+      <c r="R632" t="s">
+        <v>38</v>
+      </c>
+      <c r="S632" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="633" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B633" t="s">
+        <v>1317</v>
+      </c>
+      <c r="C633" t="s">
+        <v>1318</v>
+      </c>
+      <c r="D633" t="s">
+        <v>28</v>
+      </c>
+      <c r="E633" t="s">
+        <v>29</v>
+      </c>
+      <c r="F633" t="s">
+        <v>30</v>
+      </c>
+      <c r="G633" t="s">
+        <v>31</v>
+      </c>
+      <c r="H633" t="s">
+        <v>32</v>
+      </c>
+      <c r="I633" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J633" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K633" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L633" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M633" t="s">
+        <v>34</v>
+      </c>
+      <c r="N633" t="s">
+        <v>35</v>
+      </c>
+      <c r="O633" t="s">
+        <v>36</v>
+      </c>
+      <c r="P633" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q633" t="s">
+        <v>38</v>
+      </c>
+      <c r="R633" t="s">
+        <v>38</v>
+      </c>
+      <c r="S633" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="634" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B634" t="s">
+        <v>1319</v>
+      </c>
+      <c r="C634" t="s">
+        <v>1320</v>
+      </c>
+      <c r="D634" t="s">
+        <v>28</v>
+      </c>
+      <c r="E634" t="s">
+        <v>29</v>
+      </c>
+      <c r="F634" t="s">
+        <v>30</v>
+      </c>
+      <c r="G634" t="s">
+        <v>31</v>
+      </c>
+      <c r="H634" t="s">
+        <v>32</v>
+      </c>
+      <c r="I634" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J634" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K634" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L634" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M634" t="s">
+        <v>34</v>
+      </c>
+      <c r="N634" t="s">
+        <v>35</v>
+      </c>
+      <c r="O634" t="s">
+        <v>36</v>
+      </c>
+      <c r="P634" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q634" t="s">
+        <v>38</v>
+      </c>
+      <c r="R634" t="s">
+        <v>38</v>
+      </c>
+      <c r="S634" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="635" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B635" t="s">
+        <v>1321</v>
+      </c>
+      <c r="C635" t="s">
+        <v>1322</v>
+      </c>
+      <c r="D635" t="s">
+        <v>28</v>
+      </c>
+      <c r="E635" t="s">
+        <v>29</v>
+      </c>
+      <c r="F635" t="s">
+        <v>30</v>
+      </c>
+      <c r="G635" t="s">
+        <v>31</v>
+      </c>
+      <c r="H635" t="s">
+        <v>32</v>
+      </c>
+      <c r="I635" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J635" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K635" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L635" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M635" t="s">
+        <v>34</v>
+      </c>
+      <c r="N635" t="s">
+        <v>35</v>
+      </c>
+      <c r="O635" t="s">
+        <v>36</v>
+      </c>
+      <c r="P635" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q635" t="s">
+        <v>38</v>
+      </c>
+      <c r="R635" t="s">
+        <v>38</v>
+      </c>
+      <c r="S635" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="636" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B636" t="s">
+        <v>1323</v>
+      </c>
+      <c r="C636" t="s">
+        <v>1324</v>
+      </c>
+      <c r="D636" t="s">
+        <v>28</v>
+      </c>
+      <c r="E636" t="s">
+        <v>29</v>
+      </c>
+      <c r="F636" t="s">
+        <v>30</v>
+      </c>
+      <c r="G636" t="s">
+        <v>31</v>
+      </c>
+      <c r="H636" t="s">
+        <v>32</v>
+      </c>
+      <c r="I636" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J636" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K636" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L636" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M636" t="s">
+        <v>34</v>
+      </c>
+      <c r="N636" t="s">
+        <v>35</v>
+      </c>
+      <c r="O636" t="s">
+        <v>36</v>
+      </c>
+      <c r="P636" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q636" t="s">
+        <v>38</v>
+      </c>
+      <c r="R636" t="s">
+        <v>38</v>
+      </c>
+      <c r="S636" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="637" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B637" t="s">
+        <v>1325</v>
+      </c>
+      <c r="C637" t="s">
+        <v>1326</v>
+      </c>
+      <c r="D637" t="s">
+        <v>28</v>
+      </c>
+      <c r="E637" t="s">
+        <v>29</v>
+      </c>
+      <c r="F637" t="s">
+        <v>30</v>
+      </c>
+      <c r="G637" t="s">
+        <v>31</v>
+      </c>
+      <c r="H637" t="s">
+        <v>32</v>
+      </c>
+      <c r="I637" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J637" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K637" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L637" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M637" t="s">
+        <v>34</v>
+      </c>
+      <c r="N637" t="s">
+        <v>35</v>
+      </c>
+      <c r="O637" t="s">
+        <v>36</v>
+      </c>
+      <c r="P637" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q637" t="s">
+        <v>38</v>
+      </c>
+      <c r="R637" t="s">
+        <v>38</v>
+      </c>
+      <c r="S637" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="638" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B638" t="s">
+        <v>1327</v>
+      </c>
+      <c r="C638" t="s">
+        <v>1328</v>
+      </c>
+      <c r="D638" t="s">
+        <v>28</v>
+      </c>
+      <c r="E638" t="s">
+        <v>29</v>
+      </c>
+      <c r="F638" t="s">
+        <v>30</v>
+      </c>
+      <c r="G638" t="s">
+        <v>31</v>
+      </c>
+      <c r="H638" t="s">
+        <v>32</v>
+      </c>
+      <c r="I638" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J638" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K638" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L638" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M638" t="s">
+        <v>34</v>
+      </c>
+      <c r="N638" t="s">
+        <v>35</v>
+      </c>
+      <c r="O638" t="s">
+        <v>36</v>
+      </c>
+      <c r="P638" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q638" t="s">
+        <v>38</v>
+      </c>
+      <c r="R638" t="s">
+        <v>38</v>
+      </c>
+      <c r="S638" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="639" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B639" t="s">
+        <v>1329</v>
+      </c>
+      <c r="C639" t="s">
+        <v>1330</v>
+      </c>
+      <c r="D639" t="s">
+        <v>28</v>
+      </c>
+      <c r="E639" t="s">
+        <v>29</v>
+      </c>
+      <c r="F639" t="s">
+        <v>30</v>
+      </c>
+      <c r="G639" t="s">
+        <v>31</v>
+      </c>
+      <c r="H639" t="s">
+        <v>32</v>
+      </c>
+      <c r="I639" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J639" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K639" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L639" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M639" t="s">
+        <v>34</v>
+      </c>
+      <c r="N639" t="s">
+        <v>35</v>
+      </c>
+      <c r="O639" t="s">
+        <v>36</v>
+      </c>
+      <c r="P639" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q639" t="s">
+        <v>38</v>
+      </c>
+      <c r="R639" t="s">
+        <v>38</v>
+      </c>
+      <c r="S639" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="640" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B640" t="s">
+        <v>1331</v>
+      </c>
+      <c r="C640" t="s">
+        <v>1332</v>
+      </c>
+      <c r="D640" t="s">
+        <v>28</v>
+      </c>
+      <c r="E640" t="s">
+        <v>29</v>
+      </c>
+      <c r="F640" t="s">
+        <v>30</v>
+      </c>
+      <c r="G640" t="s">
+        <v>31</v>
+      </c>
+      <c r="H640" t="s">
+        <v>32</v>
+      </c>
+      <c r="I640" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J640" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K640" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L640" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M640" t="s">
+        <v>34</v>
+      </c>
+      <c r="N640" t="s">
+        <v>35</v>
+      </c>
+      <c r="O640" t="s">
+        <v>36</v>
+      </c>
+      <c r="P640" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q640" t="s">
+        <v>38</v>
+      </c>
+      <c r="R640" t="s">
+        <v>38</v>
+      </c>
+      <c r="S640" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="641" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B641" t="s">
+        <v>1333</v>
+      </c>
+      <c r="C641" t="s">
+        <v>1334</v>
+      </c>
+      <c r="D641" t="s">
+        <v>28</v>
+      </c>
+      <c r="E641" t="s">
+        <v>29</v>
+      </c>
+      <c r="F641" t="s">
+        <v>30</v>
+      </c>
+      <c r="G641" t="s">
+        <v>31</v>
+      </c>
+      <c r="H641" t="s">
+        <v>32</v>
+      </c>
+      <c r="I641" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J641" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K641" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L641" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M641" t="s">
+        <v>34</v>
+      </c>
+      <c r="N641" t="s">
+        <v>35</v>
+      </c>
+      <c r="O641" t="s">
+        <v>36</v>
+      </c>
+      <c r="P641" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q641" t="s">
+        <v>38</v>
+      </c>
+      <c r="R641" t="s">
+        <v>38</v>
+      </c>
+      <c r="S641" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="642" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B642" t="s">
+        <v>1335</v>
+      </c>
+      <c r="C642" t="s">
+        <v>1336</v>
+      </c>
+      <c r="D642" t="s">
+        <v>28</v>
+      </c>
+      <c r="E642" t="s">
+        <v>29</v>
+      </c>
+      <c r="F642" t="s">
+        <v>30</v>
+      </c>
+      <c r="G642" t="s">
+        <v>31</v>
+      </c>
+      <c r="H642" t="s">
+        <v>32</v>
+      </c>
+      <c r="I642" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J642" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K642" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L642" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M642" t="s">
+        <v>34</v>
+      </c>
+      <c r="N642" t="s">
+        <v>35</v>
+      </c>
+      <c r="O642" t="s">
+        <v>36</v>
+      </c>
+      <c r="P642" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q642" t="s">
+        <v>38</v>
+      </c>
+      <c r="R642" t="s">
+        <v>38</v>
+      </c>
+      <c r="S642" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="643" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B643" t="s">
+        <v>1337</v>
+      </c>
+      <c r="C643" t="s">
+        <v>1338</v>
+      </c>
+      <c r="D643" t="s">
+        <v>28</v>
+      </c>
+      <c r="E643" t="s">
+        <v>29</v>
+      </c>
+      <c r="F643" t="s">
+        <v>30</v>
+      </c>
+      <c r="G643" t="s">
+        <v>31</v>
+      </c>
+      <c r="H643" t="s">
+        <v>32</v>
+      </c>
+      <c r="I643" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J643" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K643" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L643" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M643" t="s">
+        <v>34</v>
+      </c>
+      <c r="N643" t="s">
+        <v>35</v>
+      </c>
+      <c r="O643" t="s">
+        <v>36</v>
+      </c>
+      <c r="P643" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q643" t="s">
+        <v>38</v>
+      </c>
+      <c r="R643" t="s">
+        <v>38</v>
+      </c>
+      <c r="S643" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="644" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B644" t="s">
+        <v>1339</v>
+      </c>
+      <c r="C644" t="s">
+        <v>1340</v>
+      </c>
+      <c r="D644" t="s">
+        <v>28</v>
+      </c>
+      <c r="E644" t="s">
+        <v>29</v>
+      </c>
+      <c r="F644" t="s">
+        <v>30</v>
+      </c>
+      <c r="G644" t="s">
+        <v>31</v>
+      </c>
+      <c r="H644" t="s">
+        <v>32</v>
+      </c>
+      <c r="I644" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J644" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K644" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L644" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M644" t="s">
+        <v>34</v>
+      </c>
+      <c r="N644" t="s">
+        <v>35</v>
+      </c>
+      <c r="O644" t="s">
+        <v>36</v>
+      </c>
+      <c r="P644" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q644" t="s">
+        <v>38</v>
+      </c>
+      <c r="R644" t="s">
+        <v>38</v>
+      </c>
+      <c r="S644" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="645" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B645" t="s">
+        <v>1341</v>
+      </c>
+      <c r="C645" t="s">
+        <v>1342</v>
+      </c>
+      <c r="D645" t="s">
+        <v>28</v>
+      </c>
+      <c r="E645" t="s">
+        <v>29</v>
+      </c>
+      <c r="F645" t="s">
+        <v>30</v>
+      </c>
+      <c r="G645" t="s">
+        <v>31</v>
+      </c>
+      <c r="H645" t="s">
+        <v>32</v>
+      </c>
+      <c r="I645" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J645" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K645" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L645" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M645" t="s">
+        <v>34</v>
+      </c>
+      <c r="N645" t="s">
+        <v>35</v>
+      </c>
+      <c r="O645" t="s">
+        <v>36</v>
+      </c>
+      <c r="P645" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q645" t="s">
+        <v>38</v>
+      </c>
+      <c r="R645" t="s">
+        <v>38</v>
+      </c>
+      <c r="S645" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="646" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B646" t="s">
+        <v>1343</v>
+      </c>
+      <c r="C646" t="s">
+        <v>1344</v>
+      </c>
+      <c r="D646" t="s">
+        <v>28</v>
+      </c>
+      <c r="E646" t="s">
+        <v>29</v>
+      </c>
+      <c r="F646" t="s">
+        <v>30</v>
+      </c>
+      <c r="G646" t="s">
+        <v>31</v>
+      </c>
+      <c r="H646" t="s">
+        <v>32</v>
+      </c>
+      <c r="I646" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J646" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K646" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L646" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M646" t="s">
+        <v>34</v>
+      </c>
+      <c r="N646" t="s">
+        <v>35</v>
+      </c>
+      <c r="O646" t="s">
+        <v>36</v>
+      </c>
+      <c r="P646" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q646" t="s">
+        <v>38</v>
+      </c>
+      <c r="R646" t="s">
+        <v>38</v>
+      </c>
+      <c r="S646" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="647" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B647" t="s">
+        <v>1345</v>
+      </c>
+      <c r="C647" t="s">
+        <v>1346</v>
+      </c>
+      <c r="D647" t="s">
+        <v>28</v>
+      </c>
+      <c r="E647" t="s">
+        <v>29</v>
+      </c>
+      <c r="F647" t="s">
+        <v>30</v>
+      </c>
+      <c r="G647" t="s">
+        <v>31</v>
+      </c>
+      <c r="H647" t="s">
+        <v>32</v>
+      </c>
+      <c r="I647" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J647" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K647" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L647" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M647" t="s">
+        <v>34</v>
+      </c>
+      <c r="N647" t="s">
+        <v>35</v>
+      </c>
+      <c r="O647" t="s">
+        <v>36</v>
+      </c>
+      <c r="P647" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q647" t="s">
+        <v>38</v>
+      </c>
+      <c r="R647" t="s">
+        <v>38</v>
+      </c>
+      <c r="S647" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="648" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B648" t="s">
+        <v>1347</v>
+      </c>
+      <c r="C648" t="s">
+        <v>1348</v>
+      </c>
+      <c r="D648" t="s">
+        <v>28</v>
+      </c>
+      <c r="E648" t="s">
+        <v>29</v>
+      </c>
+      <c r="F648" t="s">
+        <v>30</v>
+      </c>
+      <c r="G648" t="s">
+        <v>31</v>
+      </c>
+      <c r="H648" t="s">
+        <v>32</v>
+      </c>
+      <c r="I648" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J648" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K648" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L648" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M648" t="s">
+        <v>34</v>
+      </c>
+      <c r="N648" t="s">
+        <v>35</v>
+      </c>
+      <c r="O648" t="s">
+        <v>36</v>
+      </c>
+      <c r="P648" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q648" t="s">
+        <v>38</v>
+      </c>
+      <c r="R648" t="s">
+        <v>38</v>
+      </c>
+      <c r="S648" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="649" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B649" t="s">
+        <v>1349</v>
+      </c>
+      <c r="C649" t="s">
+        <v>1350</v>
+      </c>
+      <c r="D649" t="s">
+        <v>28</v>
+      </c>
+      <c r="E649" t="s">
+        <v>29</v>
+      </c>
+      <c r="F649" t="s">
+        <v>30</v>
+      </c>
+      <c r="G649" t="s">
+        <v>31</v>
+      </c>
+      <c r="H649" t="s">
+        <v>32</v>
+      </c>
+      <c r="I649" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J649" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K649" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L649" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M649" t="s">
+        <v>34</v>
+      </c>
+      <c r="N649" t="s">
+        <v>35</v>
+      </c>
+      <c r="O649" t="s">
+        <v>36</v>
+      </c>
+      <c r="P649" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q649" t="s">
+        <v>38</v>
+      </c>
+      <c r="R649" t="s">
+        <v>38</v>
+      </c>
+      <c r="S649" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="650" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B650" t="s">
+        <v>1351</v>
+      </c>
+      <c r="C650" t="s">
+        <v>1352</v>
+      </c>
+      <c r="D650" t="s">
+        <v>28</v>
+      </c>
+      <c r="E650" t="s">
+        <v>29</v>
+      </c>
+      <c r="F650" t="s">
+        <v>30</v>
+      </c>
+      <c r="G650" t="s">
+        <v>31</v>
+      </c>
+      <c r="H650" t="s">
+        <v>32</v>
+      </c>
+      <c r="I650" t="s">
+        <v>43</v>
+      </c>
+      <c r="J650" t="s">
+        <v>43</v>
+      </c>
+      <c r="K650" t="s">
+        <v>43</v>
+      </c>
+      <c r="L650" t="s">
+        <v>43</v>
+      </c>
+      <c r="M650" t="s">
+        <v>34</v>
+      </c>
+      <c r="N650" t="s">
+        <v>35</v>
+      </c>
+      <c r="O650" t="s">
+        <v>36</v>
+      </c>
+      <c r="P650" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q650" t="s">
+        <v>38</v>
+      </c>
+      <c r="R650" t="s">
+        <v>38</v>
+      </c>
+      <c r="S650" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="651" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B651" t="s">
+        <v>1353</v>
+      </c>
+      <c r="C651" t="s">
+        <v>1354</v>
+      </c>
+      <c r="D651" t="s">
+        <v>28</v>
+      </c>
+      <c r="E651" t="s">
+        <v>29</v>
+      </c>
+      <c r="F651" t="s">
+        <v>30</v>
+      </c>
+      <c r="G651" t="s">
+        <v>31</v>
+      </c>
+      <c r="H651" t="s">
+        <v>32</v>
+      </c>
+      <c r="I651" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J651" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K651" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L651" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M651" t="s">
+        <v>34</v>
+      </c>
+      <c r="N651" t="s">
+        <v>35</v>
+      </c>
+      <c r="O651" t="s">
+        <v>36</v>
+      </c>
+      <c r="P651" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q651" t="s">
+        <v>38</v>
+      </c>
+      <c r="R651" t="s">
+        <v>38</v>
+      </c>
+      <c r="S651" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="652" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B652" t="s">
+        <v>1355</v>
+      </c>
+      <c r="C652" t="s">
+        <v>1356</v>
+      </c>
+      <c r="D652" t="s">
+        <v>28</v>
+      </c>
+      <c r="E652" t="s">
+        <v>29</v>
+      </c>
+      <c r="F652" t="s">
+        <v>30</v>
+      </c>
+      <c r="G652" t="s">
+        <v>31</v>
+      </c>
+      <c r="H652" t="s">
+        <v>32</v>
+      </c>
+      <c r="I652" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J652" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K652" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L652" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M652" t="s">
+        <v>34</v>
+      </c>
+      <c r="N652" t="s">
+        <v>35</v>
+      </c>
+      <c r="O652" t="s">
+        <v>36</v>
+      </c>
+      <c r="P652" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q652" t="s">
+        <v>38</v>
+      </c>
+      <c r="R652" t="s">
+        <v>38</v>
+      </c>
+      <c r="S652" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="653" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B653" t="s">
+        <v>1357</v>
+      </c>
+      <c r="C653" t="s">
+        <v>1358</v>
+      </c>
+      <c r="D653" t="s">
+        <v>28</v>
+      </c>
+      <c r="E653" t="s">
+        <v>29</v>
+      </c>
+      <c r="F653" t="s">
+        <v>30</v>
+      </c>
+      <c r="G653" t="s">
+        <v>31</v>
+      </c>
+      <c r="H653" t="s">
+        <v>32</v>
+      </c>
+      <c r="I653" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J653" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K653" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L653" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M653" t="s">
+        <v>34</v>
+      </c>
+      <c r="N653" t="s">
+        <v>35</v>
+      </c>
+      <c r="O653" t="s">
+        <v>36</v>
+      </c>
+      <c r="P653" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q653" t="s">
+        <v>38</v>
+      </c>
+      <c r="R653" t="s">
+        <v>38</v>
+      </c>
+      <c r="S653" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="654" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B654" t="s">
+        <v>1359</v>
+      </c>
+      <c r="C654" t="s">
+        <v>1360</v>
+      </c>
+      <c r="D654" t="s">
+        <v>28</v>
+      </c>
+      <c r="E654" t="s">
+        <v>29</v>
+      </c>
+      <c r="F654" t="s">
+        <v>30</v>
+      </c>
+      <c r="G654" t="s">
+        <v>31</v>
+      </c>
+      <c r="H654" t="s">
+        <v>32</v>
+      </c>
+      <c r="I654" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J654" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K654" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L654" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M654" t="s">
+        <v>34</v>
+      </c>
+      <c r="N654" t="s">
+        <v>35</v>
+      </c>
+      <c r="O654" t="s">
+        <v>36</v>
+      </c>
+      <c r="P654" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q654" t="s">
+        <v>38</v>
+      </c>
+      <c r="R654" t="s">
+        <v>38</v>
+      </c>
+      <c r="S654" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="655" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B655" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C655" t="s">
+        <v>1362</v>
+      </c>
+      <c r="D655" t="s">
+        <v>28</v>
+      </c>
+      <c r="E655" t="s">
+        <v>29</v>
+      </c>
+      <c r="F655" t="s">
+        <v>30</v>
+      </c>
+      <c r="G655" t="s">
+        <v>31</v>
+      </c>
+      <c r="H655" t="s">
+        <v>32</v>
+      </c>
+      <c r="I655" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J655" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K655" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L655" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M655" t="s">
+        <v>34</v>
+      </c>
+      <c r="N655" t="s">
+        <v>35</v>
+      </c>
+      <c r="O655" t="s">
+        <v>36</v>
+      </c>
+      <c r="P655" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q655" t="s">
+        <v>38</v>
+      </c>
+      <c r="R655" t="s">
+        <v>38</v>
+      </c>
+      <c r="S655" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="656" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B656" t="s">
+        <v>1363</v>
+      </c>
+      <c r="C656" t="s">
+        <v>1364</v>
+      </c>
+      <c r="D656" t="s">
+        <v>28</v>
+      </c>
+      <c r="E656" t="s">
+        <v>29</v>
+      </c>
+      <c r="F656" t="s">
+        <v>30</v>
+      </c>
+      <c r="G656" t="s">
+        <v>31</v>
+      </c>
+      <c r="H656" t="s">
+        <v>32</v>
+      </c>
+      <c r="I656" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J656" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K656" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L656" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M656" t="s">
+        <v>34</v>
+      </c>
+      <c r="N656" t="s">
+        <v>35</v>
+      </c>
+      <c r="O656" t="s">
+        <v>36</v>
+      </c>
+      <c r="P656" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q656" t="s">
+        <v>38</v>
+      </c>
+      <c r="R656" t="s">
+        <v>38</v>
+      </c>
+      <c r="S656" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="657" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B657" t="s">
+        <v>1365</v>
+      </c>
+      <c r="C657" t="s">
+        <v>1366</v>
+      </c>
+      <c r="D657" t="s">
+        <v>28</v>
+      </c>
+      <c r="E657" t="s">
+        <v>29</v>
+      </c>
+      <c r="F657" t="s">
+        <v>30</v>
+      </c>
+      <c r="G657" t="s">
+        <v>31</v>
+      </c>
+      <c r="H657" t="s">
+        <v>32</v>
+      </c>
+      <c r="I657" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J657" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K657" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L657" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M657" t="s">
+        <v>34</v>
+      </c>
+      <c r="N657" t="s">
+        <v>35</v>
+      </c>
+      <c r="O657" t="s">
+        <v>36</v>
+      </c>
+      <c r="P657" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q657" t="s">
+        <v>38</v>
+      </c>
+      <c r="R657" t="s">
+        <v>38</v>
+      </c>
+      <c r="S657" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="658" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B658" t="s">
+        <v>1367</v>
+      </c>
+      <c r="C658" t="s">
+        <v>1368</v>
+      </c>
+      <c r="D658" t="s">
+        <v>28</v>
+      </c>
+      <c r="E658" t="s">
+        <v>29</v>
+      </c>
+      <c r="F658" t="s">
+        <v>30</v>
+      </c>
+      <c r="G658" t="s">
+        <v>31</v>
+      </c>
+      <c r="H658" t="s">
+        <v>32</v>
+      </c>
+      <c r="I658" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J658" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K658" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L658" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M658" t="s">
+        <v>34</v>
+      </c>
+      <c r="N658" t="s">
+        <v>35</v>
+      </c>
+      <c r="O658" t="s">
+        <v>36</v>
+      </c>
+      <c r="P658" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q658" t="s">
+        <v>38</v>
+      </c>
+      <c r="R658" t="s">
+        <v>38</v>
+      </c>
+      <c r="S658" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="659" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B659" t="s">
+        <v>1369</v>
+      </c>
+      <c r="C659" t="s">
+        <v>1370</v>
+      </c>
+      <c r="D659" t="s">
+        <v>28</v>
+      </c>
+      <c r="E659" t="s">
+        <v>29</v>
+      </c>
+      <c r="F659" t="s">
+        <v>30</v>
+      </c>
+      <c r="G659" t="s">
+        <v>31</v>
+      </c>
+      <c r="H659" t="s">
+        <v>32</v>
+      </c>
+      <c r="I659" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J659" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K659" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L659" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M659" t="s">
+        <v>34</v>
+      </c>
+      <c r="N659" t="s">
+        <v>35</v>
+      </c>
+      <c r="O659" t="s">
+        <v>36</v>
+      </c>
+      <c r="P659" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q659" t="s">
+        <v>38</v>
+      </c>
+      <c r="R659" t="s">
+        <v>38</v>
+      </c>
+      <c r="S659" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="660" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B660" t="s">
+        <v>1371</v>
+      </c>
+      <c r="C660" t="s">
+        <v>1372</v>
+      </c>
+      <c r="D660" t="s">
+        <v>28</v>
+      </c>
+      <c r="E660" t="s">
+        <v>29</v>
+      </c>
+      <c r="F660" t="s">
+        <v>30</v>
+      </c>
+      <c r="G660" t="s">
+        <v>31</v>
+      </c>
+      <c r="H660" t="s">
+        <v>32</v>
+      </c>
+      <c r="I660" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J660" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K660" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L660" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M660" t="s">
+        <v>34</v>
+      </c>
+      <c r="N660" t="s">
+        <v>35</v>
+      </c>
+      <c r="O660" t="s">
+        <v>36</v>
+      </c>
+      <c r="P660" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q660" t="s">
+        <v>38</v>
+      </c>
+      <c r="R660" t="s">
+        <v>38</v>
+      </c>
+      <c r="S660" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="661" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B661" t="s">
+        <v>1373</v>
+      </c>
+      <c r="C661" t="s">
+        <v>1374</v>
+      </c>
+      <c r="D661" t="s">
+        <v>28</v>
+      </c>
+      <c r="E661" t="s">
+        <v>29</v>
+      </c>
+      <c r="F661" t="s">
+        <v>30</v>
+      </c>
+      <c r="G661" t="s">
+        <v>31</v>
+      </c>
+      <c r="H661" t="s">
+        <v>32</v>
+      </c>
+      <c r="I661" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J661" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K661" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L661" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M661" t="s">
+        <v>34</v>
+      </c>
+      <c r="N661" t="s">
+        <v>35</v>
+      </c>
+      <c r="O661" t="s">
+        <v>36</v>
+      </c>
+      <c r="P661" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q661" t="s">
+        <v>38</v>
+      </c>
+      <c r="R661" t="s">
+        <v>38</v>
+      </c>
+      <c r="S661" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="662" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B662" t="s">
+        <v>1375</v>
+      </c>
+      <c r="C662" t="s">
+        <v>1376</v>
+      </c>
+      <c r="D662" t="s">
+        <v>28</v>
+      </c>
+      <c r="E662" t="s">
+        <v>29</v>
+      </c>
+      <c r="F662" t="s">
+        <v>30</v>
+      </c>
+      <c r="G662" t="s">
+        <v>31</v>
+      </c>
+      <c r="H662" t="s">
+        <v>32</v>
+      </c>
+      <c r="I662" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J662" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K662" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L662" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M662" t="s">
+        <v>34</v>
+      </c>
+      <c r="N662" t="s">
+        <v>35</v>
+      </c>
+      <c r="O662" t="s">
+        <v>36</v>
+      </c>
+      <c r="P662" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q662" t="s">
+        <v>38</v>
+      </c>
+      <c r="R662" t="s">
+        <v>38</v>
+      </c>
+      <c r="S662" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="663" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B663" t="s">
+        <v>1377</v>
+      </c>
+      <c r="C663" t="s">
+        <v>1378</v>
+      </c>
+      <c r="D663" t="s">
+        <v>28</v>
+      </c>
+      <c r="E663" t="s">
+        <v>29</v>
+      </c>
+      <c r="F663" t="s">
+        <v>30</v>
+      </c>
+      <c r="G663" t="s">
+        <v>31</v>
+      </c>
+      <c r="H663" t="s">
+        <v>32</v>
+      </c>
+      <c r="I663" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J663" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K663" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L663" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M663" t="s">
+        <v>34</v>
+      </c>
+      <c r="N663" t="s">
+        <v>35</v>
+      </c>
+      <c r="O663" t="s">
+        <v>36</v>
+      </c>
+      <c r="P663" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q663" t="s">
+        <v>38</v>
+      </c>
+      <c r="R663" t="s">
+        <v>38</v>
+      </c>
+      <c r="S663" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="664" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B664" t="s">
+        <v>1379</v>
+      </c>
+      <c r="C664" t="s">
+        <v>1380</v>
+      </c>
+      <c r="D664" t="s">
+        <v>28</v>
+      </c>
+      <c r="E664" t="s">
+        <v>29</v>
+      </c>
+      <c r="F664" t="s">
+        <v>30</v>
+      </c>
+      <c r="G664" t="s">
+        <v>31</v>
+      </c>
+      <c r="H664" t="s">
+        <v>32</v>
+      </c>
+      <c r="I664" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J664" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K664" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L664" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M664" t="s">
+        <v>34</v>
+      </c>
+      <c r="N664" t="s">
+        <v>35</v>
+      </c>
+      <c r="O664" t="s">
+        <v>36</v>
+      </c>
+      <c r="P664" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q664" t="s">
+        <v>38</v>
+      </c>
+      <c r="R664" t="s">
+        <v>38</v>
+      </c>
+      <c r="S664" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="665" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B665" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C665" t="s">
+        <v>1382</v>
+      </c>
+      <c r="D665" t="s">
+        <v>28</v>
+      </c>
+      <c r="E665" t="s">
+        <v>29</v>
+      </c>
+      <c r="F665" t="s">
+        <v>30</v>
+      </c>
+      <c r="G665" t="s">
+        <v>31</v>
+      </c>
+      <c r="H665" t="s">
+        <v>32</v>
+      </c>
+      <c r="I665" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J665" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K665" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L665" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M665" t="s">
+        <v>34</v>
+      </c>
+      <c r="N665" t="s">
+        <v>35</v>
+      </c>
+      <c r="O665" t="s">
+        <v>36</v>
+      </c>
+      <c r="P665" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q665" t="s">
+        <v>38</v>
+      </c>
+      <c r="R665" t="s">
+        <v>38</v>
+      </c>
+      <c r="S665" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="666" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B666" t="s">
+        <v>1383</v>
+      </c>
+      <c r="C666" t="s">
+        <v>1384</v>
+      </c>
+      <c r="D666" t="s">
+        <v>28</v>
+      </c>
+      <c r="E666" t="s">
+        <v>29</v>
+      </c>
+      <c r="F666" t="s">
+        <v>30</v>
+      </c>
+      <c r="G666" t="s">
+        <v>31</v>
+      </c>
+      <c r="H666" t="s">
+        <v>32</v>
+      </c>
+      <c r="I666" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J666" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K666" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L666" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M666" t="s">
+        <v>34</v>
+      </c>
+      <c r="N666" t="s">
+        <v>35</v>
+      </c>
+      <c r="O666" t="s">
+        <v>36</v>
+      </c>
+      <c r="P666" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q666" t="s">
+        <v>38</v>
+      </c>
+      <c r="R666" t="s">
+        <v>38</v>
+      </c>
+      <c r="S666" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="667" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B667" t="s">
+        <v>1385</v>
+      </c>
+      <c r="C667" t="s">
+        <v>1386</v>
+      </c>
+      <c r="D667" t="s">
+        <v>28</v>
+      </c>
+      <c r="E667" t="s">
+        <v>29</v>
+      </c>
+      <c r="F667" t="s">
+        <v>30</v>
+      </c>
+      <c r="G667" t="s">
+        <v>31</v>
+      </c>
+      <c r="H667" t="s">
+        <v>32</v>
+      </c>
+      <c r="I667" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J667" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K667" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L667" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M667" t="s">
+        <v>34</v>
+      </c>
+      <c r="N667" t="s">
+        <v>35</v>
+      </c>
+      <c r="O667" t="s">
+        <v>36</v>
+      </c>
+      <c r="P667" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q667" t="s">
+        <v>38</v>
+      </c>
+      <c r="R667" t="s">
+        <v>38</v>
+      </c>
+      <c r="S667" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="668" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B668" t="s">
+        <v>1387</v>
+      </c>
+      <c r="C668" t="s">
+        <v>1388</v>
+      </c>
+      <c r="D668" t="s">
+        <v>28</v>
+      </c>
+      <c r="E668" t="s">
+        <v>29</v>
+      </c>
+      <c r="F668" t="s">
+        <v>30</v>
+      </c>
+      <c r="G668" t="s">
+        <v>31</v>
+      </c>
+      <c r="H668" t="s">
+        <v>32</v>
+      </c>
+      <c r="I668" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J668" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K668" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L668" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M668" t="s">
+        <v>34</v>
+      </c>
+      <c r="N668" t="s">
+        <v>35</v>
+      </c>
+      <c r="O668" t="s">
+        <v>36</v>
+      </c>
+      <c r="P668" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q668" t="s">
+        <v>38</v>
+      </c>
+      <c r="R668" t="s">
+        <v>38</v>
+      </c>
+      <c r="S668" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="669" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B669" t="s">
+        <v>1389</v>
+      </c>
+      <c r="C669" t="s">
+        <v>1390</v>
+      </c>
+      <c r="D669" t="s">
+        <v>28</v>
+      </c>
+      <c r="E669" t="s">
+        <v>29</v>
+      </c>
+      <c r="F669" t="s">
+        <v>30</v>
+      </c>
+      <c r="G669" t="s">
+        <v>31</v>
+      </c>
+      <c r="H669" t="s">
+        <v>32</v>
+      </c>
+      <c r="I669" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J669" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K669" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L669" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M669" t="s">
+        <v>34</v>
+      </c>
+      <c r="N669" t="s">
+        <v>35</v>
+      </c>
+      <c r="O669" t="s">
+        <v>36</v>
+      </c>
+      <c r="P669" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q669" t="s">
+        <v>38</v>
+      </c>
+      <c r="R669" t="s">
+        <v>38</v>
+      </c>
+      <c r="S669" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="670" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B670" t="s">
+        <v>1391</v>
+      </c>
+      <c r="C670" t="s">
+        <v>1392</v>
+      </c>
+      <c r="D670" t="s">
+        <v>28</v>
+      </c>
+      <c r="E670" t="s">
+        <v>29</v>
+      </c>
+      <c r="F670" t="s">
+        <v>30</v>
+      </c>
+      <c r="G670" t="s">
+        <v>31</v>
+      </c>
+      <c r="H670" t="s">
+        <v>32</v>
+      </c>
+      <c r="I670" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J670" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K670" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L670" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M670" t="s">
+        <v>34</v>
+      </c>
+      <c r="N670" t="s">
+        <v>35</v>
+      </c>
+      <c r="O670" t="s">
+        <v>36</v>
+      </c>
+      <c r="P670" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q670" t="s">
+        <v>38</v>
+      </c>
+      <c r="R670" t="s">
+        <v>38</v>
+      </c>
+      <c r="S670" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="671" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B671" t="s">
+        <v>1393</v>
+      </c>
+      <c r="C671" t="s">
+        <v>1394</v>
+      </c>
+      <c r="D671" t="s">
+        <v>28</v>
+      </c>
+      <c r="E671" t="s">
+        <v>29</v>
+      </c>
+      <c r="F671" t="s">
+        <v>30</v>
+      </c>
+      <c r="G671" t="s">
+        <v>31</v>
+      </c>
+      <c r="H671" t="s">
+        <v>32</v>
+      </c>
+      <c r="I671" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J671" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K671" t="s">
+        <v>1284</v>
+      </c>
+      <c r="L671" t="s">
+        <v>1284</v>
+      </c>
+      <c r="M671" t="s">
+        <v>34</v>
+      </c>
+      <c r="N671" t="s">
+        <v>35</v>
+      </c>
+      <c r="O671" t="s">
+        <v>36</v>
+      </c>
+      <c r="P671" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q671" t="s">
+        <v>38</v>
+      </c>
+      <c r="R671" t="s">
+        <v>38</v>
+      </c>
+      <c r="S671" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: update session ID and last run date in config.json; update backup Excel files
</commit_message>
<xml_diff>
--- a/py_test_ui/EXCEL FILE/backuprecordCal_PM.xlsx
+++ b/py_test_ui/EXCEL FILE/backuprecordCal_PM.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\forms-1\py_test_ui\EXCEL FILE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_50ED3F369565C60E62355476585DCE3A874AAE20" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{088EA6BC-0A22-42A6-A4B9-B3E7F58B807C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Z$718</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13314" uniqueCount="1395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14363" uniqueCount="1490">
   <si>
     <t>N0</t>
   </si>
@@ -4205,6 +4208,291 @@
   </si>
   <si>
     <t>PYT3D_02584</t>
+  </si>
+  <si>
+    <t>310393</t>
+  </si>
+  <si>
+    <t>PYT3_08132</t>
+  </si>
+  <si>
+    <t>26/06/2026</t>
+  </si>
+  <si>
+    <t>354462</t>
+  </si>
+  <si>
+    <t>PYT3_08627</t>
+  </si>
+  <si>
+    <t>398773</t>
+  </si>
+  <si>
+    <t>PYT3_09220</t>
+  </si>
+  <si>
+    <t>398779</t>
+  </si>
+  <si>
+    <t>PYT3_09223</t>
+  </si>
+  <si>
+    <t>398905</t>
+  </si>
+  <si>
+    <t>PYT3_09224</t>
+  </si>
+  <si>
+    <t>398906</t>
+  </si>
+  <si>
+    <t>PYT3_09225</t>
+  </si>
+  <si>
+    <t>398908</t>
+  </si>
+  <si>
+    <t>PYT3_09227</t>
+  </si>
+  <si>
+    <t>428314</t>
+  </si>
+  <si>
+    <t>PYT3_10046</t>
+  </si>
+  <si>
+    <t>428315</t>
+  </si>
+  <si>
+    <t>PYT3_10047</t>
+  </si>
+  <si>
+    <t>428316</t>
+  </si>
+  <si>
+    <t>PYT3_10048</t>
+  </si>
+  <si>
+    <t>428317</t>
+  </si>
+  <si>
+    <t>PYT3_10049</t>
+  </si>
+  <si>
+    <t>428318</t>
+  </si>
+  <si>
+    <t>PYT3_10050</t>
+  </si>
+  <si>
+    <t>40561</t>
+  </si>
+  <si>
+    <t>PYT3_02958</t>
+  </si>
+  <si>
+    <t>402289</t>
+  </si>
+  <si>
+    <t>PYT3_09309</t>
+  </si>
+  <si>
+    <t>405975</t>
+  </si>
+  <si>
+    <t>PYT3_09437</t>
+  </si>
+  <si>
+    <t>379743</t>
+  </si>
+  <si>
+    <t>PYT3T_09065</t>
+  </si>
+  <si>
+    <t>146987</t>
+  </si>
+  <si>
+    <t>PYT3D_05348</t>
+  </si>
+  <si>
+    <t>40162</t>
+  </si>
+  <si>
+    <t>PYT3_02569</t>
+  </si>
+  <si>
+    <t>292449</t>
+  </si>
+  <si>
+    <t>PYT3_07669</t>
+  </si>
+  <si>
+    <t>408024</t>
+  </si>
+  <si>
+    <t>PYT3_09495</t>
+  </si>
+  <si>
+    <t>37561</t>
+  </si>
+  <si>
+    <t>PYT3_01335</t>
+  </si>
+  <si>
+    <t>37666</t>
+  </si>
+  <si>
+    <t>PYT3_01440</t>
+  </si>
+  <si>
+    <t>260583</t>
+  </si>
+  <si>
+    <t>PYT3_07100</t>
+  </si>
+  <si>
+    <t>389785</t>
+  </si>
+  <si>
+    <t>PYT3_09160</t>
+  </si>
+  <si>
+    <t>396363</t>
+  </si>
+  <si>
+    <t>PYT3_09182</t>
+  </si>
+  <si>
+    <t>290406</t>
+  </si>
+  <si>
+    <t>PYT3T_07644</t>
+  </si>
+  <si>
+    <t>36478</t>
+  </si>
+  <si>
+    <t>PYT3_01148</t>
+  </si>
+  <si>
+    <t>147124</t>
+  </si>
+  <si>
+    <t>PYT3_05485</t>
+  </si>
+  <si>
+    <t>40422</t>
+  </si>
+  <si>
+    <t>PYT3_02819</t>
+  </si>
+  <si>
+    <t>216616</t>
+  </si>
+  <si>
+    <t>PYT3_06541</t>
+  </si>
+  <si>
+    <t>216634</t>
+  </si>
+  <si>
+    <t>PYT3_06559</t>
+  </si>
+  <si>
+    <t>237278</t>
+  </si>
+  <si>
+    <t>PYT3_06785</t>
+  </si>
+  <si>
+    <t>237279</t>
+  </si>
+  <si>
+    <t>PYT3_06786</t>
+  </si>
+  <si>
+    <t>425949</t>
+  </si>
+  <si>
+    <t>PYT3_09963</t>
+  </si>
+  <si>
+    <t>425953</t>
+  </si>
+  <si>
+    <t>PYT3_09967</t>
+  </si>
+  <si>
+    <t>434474</t>
+  </si>
+  <si>
+    <t>PYT3_10207</t>
+  </si>
+  <si>
+    <t>434475</t>
+  </si>
+  <si>
+    <t>PYT3_10208</t>
+  </si>
+  <si>
+    <t>147131</t>
+  </si>
+  <si>
+    <t>PYT3_05492</t>
+  </si>
+  <si>
+    <t>425933</t>
+  </si>
+  <si>
+    <t>PYT3_09947</t>
+  </si>
+  <si>
+    <t>38819</t>
+  </si>
+  <si>
+    <t>PYT3_02291</t>
+  </si>
+  <si>
+    <t>375696</t>
+  </si>
+  <si>
+    <t>PYT3_08995</t>
+  </si>
+  <si>
+    <t>179412</t>
+  </si>
+  <si>
+    <t>PYT3_05854</t>
+  </si>
+  <si>
+    <t>38147</t>
+  </si>
+  <si>
+    <t>PYT3_01920</t>
+  </si>
+  <si>
+    <t>323432</t>
+  </si>
+  <si>
+    <t>PYT3D_08374</t>
+  </si>
+  <si>
+    <t>37913</t>
+  </si>
+  <si>
+    <t>PYT3_01687</t>
+  </si>
+  <si>
+    <t>237194</t>
+  </si>
+  <si>
+    <t>PYT3_06701</t>
+  </si>
+  <si>
+    <t>40259</t>
+  </si>
+  <si>
+    <t>PYT3_02666</t>
   </si>
 </sst>
 </file>
@@ -4223,7 +4511,6 @@
       <b/>
       <sz val="11"/>
       <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -4568,8 +4855,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z671"/>
+  <dimension ref="A1:Z718"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="16.296875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -42774,6 +43064,12 @@
       <c r="S616" t="s">
         <v>39</v>
       </c>
+      <c r="V616" t="s">
+        <v>40</v>
+      </c>
+      <c r="W616" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="617" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B617" t="s">
@@ -42830,6 +43126,12 @@
       <c r="S617" t="s">
         <v>39</v>
       </c>
+      <c r="V617" t="s">
+        <v>40</v>
+      </c>
+      <c r="W617" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="618" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B618" t="s">
@@ -42886,6 +43188,12 @@
       <c r="S618" t="s">
         <v>39</v>
       </c>
+      <c r="V618" t="s">
+        <v>40</v>
+      </c>
+      <c r="W618" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="619" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B619" t="s">
@@ -42942,6 +43250,12 @@
       <c r="S619" t="s">
         <v>39</v>
       </c>
+      <c r="V619" t="s">
+        <v>40</v>
+      </c>
+      <c r="W619" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="620" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B620" t="s">
@@ -42998,6 +43312,12 @@
       <c r="S620" t="s">
         <v>39</v>
       </c>
+      <c r="V620" t="s">
+        <v>40</v>
+      </c>
+      <c r="W620" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="621" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B621" t="s">
@@ -43054,6 +43374,12 @@
       <c r="S621" t="s">
         <v>39</v>
       </c>
+      <c r="V621" t="s">
+        <v>40</v>
+      </c>
+      <c r="W621" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="622" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B622" t="s">
@@ -43110,6 +43436,12 @@
       <c r="S622" t="s">
         <v>39</v>
       </c>
+      <c r="V622" t="s">
+        <v>40</v>
+      </c>
+      <c r="W622" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="623" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B623" t="s">
@@ -43166,6 +43498,12 @@
       <c r="S623" t="s">
         <v>39</v>
       </c>
+      <c r="V623" t="s">
+        <v>40</v>
+      </c>
+      <c r="W623" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="624" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B624" t="s">
@@ -43222,8 +43560,14 @@
       <c r="S624" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="625" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V624" t="s">
+        <v>40</v>
+      </c>
+      <c r="W624" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="625" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B625" t="s">
         <v>1301</v>
       </c>
@@ -43278,8 +43622,14 @@
       <c r="S625" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="626" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V625" t="s">
+        <v>40</v>
+      </c>
+      <c r="W625" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="626" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B626" t="s">
         <v>1303</v>
       </c>
@@ -43334,8 +43684,14 @@
       <c r="S626" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="627" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V626" t="s">
+        <v>40</v>
+      </c>
+      <c r="W626" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="627" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B627" t="s">
         <v>1305</v>
       </c>
@@ -43390,8 +43746,14 @@
       <c r="S627" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="628" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V627" t="s">
+        <v>40</v>
+      </c>
+      <c r="W627" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="628" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B628" t="s">
         <v>1307</v>
       </c>
@@ -43446,8 +43808,14 @@
       <c r="S628" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="629" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V628" t="s">
+        <v>40</v>
+      </c>
+      <c r="W628" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="629" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B629" t="s">
         <v>1309</v>
       </c>
@@ -43502,8 +43870,14 @@
       <c r="S629" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="630" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V629" t="s">
+        <v>40</v>
+      </c>
+      <c r="W629" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="630" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B630" t="s">
         <v>1311</v>
       </c>
@@ -43558,8 +43932,14 @@
       <c r="S630" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="631" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V630" t="s">
+        <v>40</v>
+      </c>
+      <c r="W630" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="631" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B631" t="s">
         <v>1313</v>
       </c>
@@ -43614,8 +43994,14 @@
       <c r="S631" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="632" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V631" t="s">
+        <v>40</v>
+      </c>
+      <c r="W631" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="632" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B632" t="s">
         <v>1315</v>
       </c>
@@ -43670,8 +44056,14 @@
       <c r="S632" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="633" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V632" t="s">
+        <v>40</v>
+      </c>
+      <c r="W632" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="633" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B633" t="s">
         <v>1317</v>
       </c>
@@ -43726,8 +44118,14 @@
       <c r="S633" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="634" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V633" t="s">
+        <v>40</v>
+      </c>
+      <c r="W633" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="634" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B634" t="s">
         <v>1319</v>
       </c>
@@ -43782,8 +44180,14 @@
       <c r="S634" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="635" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V634" t="s">
+        <v>40</v>
+      </c>
+      <c r="W634" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="635" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B635" t="s">
         <v>1321</v>
       </c>
@@ -43838,8 +44242,14 @@
       <c r="S635" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="636" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V635" t="s">
+        <v>40</v>
+      </c>
+      <c r="W635" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="636" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B636" t="s">
         <v>1323</v>
       </c>
@@ -43894,8 +44304,14 @@
       <c r="S636" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="637" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V636" t="s">
+        <v>40</v>
+      </c>
+      <c r="W636" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="637" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B637" t="s">
         <v>1325</v>
       </c>
@@ -43950,8 +44366,14 @@
       <c r="S637" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="638" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V637" t="s">
+        <v>40</v>
+      </c>
+      <c r="W637" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="638" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B638" t="s">
         <v>1327</v>
       </c>
@@ -44006,8 +44428,14 @@
       <c r="S638" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="639" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V638" t="s">
+        <v>40</v>
+      </c>
+      <c r="W638" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="639" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B639" t="s">
         <v>1329</v>
       </c>
@@ -44062,8 +44490,14 @@
       <c r="S639" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="640" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V639" t="s">
+        <v>40</v>
+      </c>
+      <c r="W639" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="640" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B640" t="s">
         <v>1331</v>
       </c>
@@ -44118,8 +44552,14 @@
       <c r="S640" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="641" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V640" t="s">
+        <v>40</v>
+      </c>
+      <c r="W640" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="641" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B641" t="s">
         <v>1333</v>
       </c>
@@ -44174,8 +44614,14 @@
       <c r="S641" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="642" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V641" t="s">
+        <v>40</v>
+      </c>
+      <c r="W641" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="642" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B642" t="s">
         <v>1335</v>
       </c>
@@ -44230,8 +44676,14 @@
       <c r="S642" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="643" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V642" t="s">
+        <v>40</v>
+      </c>
+      <c r="W642" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="643" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B643" t="s">
         <v>1337</v>
       </c>
@@ -44286,8 +44738,14 @@
       <c r="S643" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="644" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V643" t="s">
+        <v>40</v>
+      </c>
+      <c r="W643" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="644" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B644" t="s">
         <v>1339</v>
       </c>
@@ -44342,8 +44800,14 @@
       <c r="S644" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="645" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V644" t="s">
+        <v>40</v>
+      </c>
+      <c r="W644" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="645" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B645" t="s">
         <v>1341</v>
       </c>
@@ -44398,8 +44862,14 @@
       <c r="S645" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="646" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V645" t="s">
+        <v>40</v>
+      </c>
+      <c r="W645" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="646" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B646" t="s">
         <v>1343</v>
       </c>
@@ -44454,8 +44924,14 @@
       <c r="S646" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="647" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V646" t="s">
+        <v>40</v>
+      </c>
+      <c r="W646" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="647" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B647" t="s">
         <v>1345</v>
       </c>
@@ -44510,8 +44986,14 @@
       <c r="S647" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="648" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V647" t="s">
+        <v>40</v>
+      </c>
+      <c r="W647" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="648" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B648" t="s">
         <v>1347</v>
       </c>
@@ -44566,8 +45048,14 @@
       <c r="S648" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="649" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V648" t="s">
+        <v>40</v>
+      </c>
+      <c r="W648" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="649" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B649" t="s">
         <v>1349</v>
       </c>
@@ -44622,8 +45110,14 @@
       <c r="S649" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="650" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V649" t="s">
+        <v>40</v>
+      </c>
+      <c r="W649" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="650" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B650" t="s">
         <v>1351</v>
       </c>
@@ -44678,8 +45172,14 @@
       <c r="S650" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="651" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V650" t="s">
+        <v>40</v>
+      </c>
+      <c r="W650" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="651" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B651" t="s">
         <v>1353</v>
       </c>
@@ -44734,8 +45234,14 @@
       <c r="S651" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="652" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V651" t="s">
+        <v>40</v>
+      </c>
+      <c r="W651" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="652" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B652" t="s">
         <v>1355</v>
       </c>
@@ -44790,8 +45296,14 @@
       <c r="S652" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="653" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V652" t="s">
+        <v>40</v>
+      </c>
+      <c r="W652" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="653" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B653" t="s">
         <v>1357</v>
       </c>
@@ -44846,8 +45358,14 @@
       <c r="S653" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="654" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V653" t="s">
+        <v>40</v>
+      </c>
+      <c r="W653" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="654" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B654" t="s">
         <v>1359</v>
       </c>
@@ -44902,8 +45420,14 @@
       <c r="S654" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="655" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V654" t="s">
+        <v>40</v>
+      </c>
+      <c r="W654" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="655" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B655" t="s">
         <v>1361</v>
       </c>
@@ -44958,8 +45482,14 @@
       <c r="S655" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="656" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V655" t="s">
+        <v>40</v>
+      </c>
+      <c r="W655" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="656" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B656" t="s">
         <v>1363</v>
       </c>
@@ -45014,8 +45544,14 @@
       <c r="S656" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="657" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V656" t="s">
+        <v>40</v>
+      </c>
+      <c r="W656" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="657" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B657" t="s">
         <v>1365</v>
       </c>
@@ -45070,8 +45606,14 @@
       <c r="S657" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="658" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V657" t="s">
+        <v>40</v>
+      </c>
+      <c r="W657" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="658" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B658" t="s">
         <v>1367</v>
       </c>
@@ -45126,8 +45668,14 @@
       <c r="S658" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="659" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V658" t="s">
+        <v>40</v>
+      </c>
+      <c r="W658" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="659" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B659" t="s">
         <v>1369</v>
       </c>
@@ -45182,8 +45730,14 @@
       <c r="S659" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="660" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V659" t="s">
+        <v>40</v>
+      </c>
+      <c r="W659" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="660" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B660" t="s">
         <v>1371</v>
       </c>
@@ -45238,8 +45792,14 @@
       <c r="S660" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="661" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V660" t="s">
+        <v>40</v>
+      </c>
+      <c r="W660" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="661" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B661" t="s">
         <v>1373</v>
       </c>
@@ -45294,8 +45854,14 @@
       <c r="S661" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="662" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V661" t="s">
+        <v>40</v>
+      </c>
+      <c r="W661" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="662" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B662" t="s">
         <v>1375</v>
       </c>
@@ -45350,8 +45916,14 @@
       <c r="S662" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="663" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V662" t="s">
+        <v>40</v>
+      </c>
+      <c r="W662" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="663" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B663" t="s">
         <v>1377</v>
       </c>
@@ -45406,8 +45978,14 @@
       <c r="S663" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="664" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V663" t="s">
+        <v>40</v>
+      </c>
+      <c r="W663" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="664" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B664" t="s">
         <v>1379</v>
       </c>
@@ -45462,8 +46040,14 @@
       <c r="S664" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="665" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V664" t="s">
+        <v>40</v>
+      </c>
+      <c r="W664" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="665" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B665" t="s">
         <v>1381</v>
       </c>
@@ -45518,8 +46102,14 @@
       <c r="S665" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="666" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V665" t="s">
+        <v>40</v>
+      </c>
+      <c r="W665" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="666" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B666" t="s">
         <v>1383</v>
       </c>
@@ -45574,8 +46164,14 @@
       <c r="S666" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="667" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V666" t="s">
+        <v>40</v>
+      </c>
+      <c r="W666" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="667" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B667" t="s">
         <v>1385</v>
       </c>
@@ -45630,8 +46226,14 @@
       <c r="S667" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="668" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V667" t="s">
+        <v>40</v>
+      </c>
+      <c r="W667" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="668" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B668" t="s">
         <v>1387</v>
       </c>
@@ -45686,8 +46288,14 @@
       <c r="S668" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="669" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V668" t="s">
+        <v>40</v>
+      </c>
+      <c r="W668" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="669" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B669" t="s">
         <v>1389</v>
       </c>
@@ -45742,8 +46350,14 @@
       <c r="S669" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="670" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V669" t="s">
+        <v>40</v>
+      </c>
+      <c r="W669" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="670" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B670" t="s">
         <v>1391</v>
       </c>
@@ -45798,8 +46412,14 @@
       <c r="S670" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="671" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="V670" t="s">
+        <v>40</v>
+      </c>
+      <c r="W670" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="671" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B671" t="s">
         <v>1393</v>
       </c>
@@ -45853,6 +46473,2917 @@
       </c>
       <c r="S671" t="s">
         <v>39</v>
+      </c>
+      <c r="V671" t="s">
+        <v>40</v>
+      </c>
+      <c r="W671" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="672" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B672" t="s">
+        <v>1395</v>
+      </c>
+      <c r="C672" t="s">
+        <v>1396</v>
+      </c>
+      <c r="D672" t="s">
+        <v>28</v>
+      </c>
+      <c r="E672" t="s">
+        <v>29</v>
+      </c>
+      <c r="F672" t="s">
+        <v>30</v>
+      </c>
+      <c r="G672" t="s">
+        <v>31</v>
+      </c>
+      <c r="H672" t="s">
+        <v>32</v>
+      </c>
+      <c r="I672" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J672" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K672" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L672" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M672" t="s">
+        <v>34</v>
+      </c>
+      <c r="N672" t="s">
+        <v>35</v>
+      </c>
+      <c r="O672" t="s">
+        <v>36</v>
+      </c>
+      <c r="P672" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q672" t="s">
+        <v>38</v>
+      </c>
+      <c r="R672" t="s">
+        <v>38</v>
+      </c>
+      <c r="S672" t="s">
+        <v>39</v>
+      </c>
+      <c r="V672" t="s">
+        <v>40</v>
+      </c>
+      <c r="W672" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="673" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B673" t="s">
+        <v>1398</v>
+      </c>
+      <c r="C673" t="s">
+        <v>1399</v>
+      </c>
+      <c r="D673" t="s">
+        <v>28</v>
+      </c>
+      <c r="E673" t="s">
+        <v>29</v>
+      </c>
+      <c r="F673" t="s">
+        <v>30</v>
+      </c>
+      <c r="G673" t="s">
+        <v>31</v>
+      </c>
+      <c r="H673" t="s">
+        <v>32</v>
+      </c>
+      <c r="I673" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J673" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K673" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L673" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M673" t="s">
+        <v>34</v>
+      </c>
+      <c r="N673" t="s">
+        <v>35</v>
+      </c>
+      <c r="O673" t="s">
+        <v>36</v>
+      </c>
+      <c r="P673" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q673" t="s">
+        <v>38</v>
+      </c>
+      <c r="R673" t="s">
+        <v>38</v>
+      </c>
+      <c r="S673" t="s">
+        <v>39</v>
+      </c>
+      <c r="V673" t="s">
+        <v>40</v>
+      </c>
+      <c r="W673" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="674" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B674" t="s">
+        <v>1400</v>
+      </c>
+      <c r="C674" t="s">
+        <v>1401</v>
+      </c>
+      <c r="D674" t="s">
+        <v>28</v>
+      </c>
+      <c r="E674" t="s">
+        <v>29</v>
+      </c>
+      <c r="F674" t="s">
+        <v>30</v>
+      </c>
+      <c r="G674" t="s">
+        <v>31</v>
+      </c>
+      <c r="H674" t="s">
+        <v>32</v>
+      </c>
+      <c r="I674" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J674" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K674" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L674" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M674" t="s">
+        <v>34</v>
+      </c>
+      <c r="N674" t="s">
+        <v>35</v>
+      </c>
+      <c r="O674" t="s">
+        <v>36</v>
+      </c>
+      <c r="P674" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q674" t="s">
+        <v>38</v>
+      </c>
+      <c r="R674" t="s">
+        <v>38</v>
+      </c>
+      <c r="S674" t="s">
+        <v>39</v>
+      </c>
+      <c r="V674" t="s">
+        <v>40</v>
+      </c>
+      <c r="W674" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="675" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B675" t="s">
+        <v>1402</v>
+      </c>
+      <c r="C675" t="s">
+        <v>1403</v>
+      </c>
+      <c r="D675" t="s">
+        <v>28</v>
+      </c>
+      <c r="E675" t="s">
+        <v>29</v>
+      </c>
+      <c r="F675" t="s">
+        <v>30</v>
+      </c>
+      <c r="G675" t="s">
+        <v>31</v>
+      </c>
+      <c r="H675" t="s">
+        <v>32</v>
+      </c>
+      <c r="I675" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J675" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K675" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L675" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M675" t="s">
+        <v>34</v>
+      </c>
+      <c r="N675" t="s">
+        <v>35</v>
+      </c>
+      <c r="O675" t="s">
+        <v>36</v>
+      </c>
+      <c r="P675" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q675" t="s">
+        <v>38</v>
+      </c>
+      <c r="R675" t="s">
+        <v>38</v>
+      </c>
+      <c r="S675" t="s">
+        <v>39</v>
+      </c>
+      <c r="V675" t="s">
+        <v>40</v>
+      </c>
+      <c r="W675" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="676" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B676" t="s">
+        <v>1404</v>
+      </c>
+      <c r="C676" t="s">
+        <v>1405</v>
+      </c>
+      <c r="D676" t="s">
+        <v>28</v>
+      </c>
+      <c r="E676" t="s">
+        <v>29</v>
+      </c>
+      <c r="F676" t="s">
+        <v>30</v>
+      </c>
+      <c r="G676" t="s">
+        <v>31</v>
+      </c>
+      <c r="H676" t="s">
+        <v>32</v>
+      </c>
+      <c r="I676" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J676" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K676" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L676" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M676" t="s">
+        <v>34</v>
+      </c>
+      <c r="N676" t="s">
+        <v>35</v>
+      </c>
+      <c r="O676" t="s">
+        <v>36</v>
+      </c>
+      <c r="P676" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q676" t="s">
+        <v>38</v>
+      </c>
+      <c r="R676" t="s">
+        <v>38</v>
+      </c>
+      <c r="S676" t="s">
+        <v>39</v>
+      </c>
+      <c r="V676" t="s">
+        <v>40</v>
+      </c>
+      <c r="W676" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="677" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B677" t="s">
+        <v>1406</v>
+      </c>
+      <c r="C677" t="s">
+        <v>1407</v>
+      </c>
+      <c r="D677" t="s">
+        <v>28</v>
+      </c>
+      <c r="E677" t="s">
+        <v>29</v>
+      </c>
+      <c r="F677" t="s">
+        <v>30</v>
+      </c>
+      <c r="G677" t="s">
+        <v>31</v>
+      </c>
+      <c r="H677" t="s">
+        <v>32</v>
+      </c>
+      <c r="I677" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J677" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K677" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L677" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M677" t="s">
+        <v>34</v>
+      </c>
+      <c r="N677" t="s">
+        <v>35</v>
+      </c>
+      <c r="O677" t="s">
+        <v>36</v>
+      </c>
+      <c r="P677" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q677" t="s">
+        <v>38</v>
+      </c>
+      <c r="R677" t="s">
+        <v>38</v>
+      </c>
+      <c r="S677" t="s">
+        <v>39</v>
+      </c>
+      <c r="V677" t="s">
+        <v>40</v>
+      </c>
+      <c r="W677" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="678" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B678" t="s">
+        <v>1408</v>
+      </c>
+      <c r="C678" t="s">
+        <v>1409</v>
+      </c>
+      <c r="D678" t="s">
+        <v>28</v>
+      </c>
+      <c r="E678" t="s">
+        <v>29</v>
+      </c>
+      <c r="F678" t="s">
+        <v>30</v>
+      </c>
+      <c r="G678" t="s">
+        <v>31</v>
+      </c>
+      <c r="H678" t="s">
+        <v>32</v>
+      </c>
+      <c r="I678" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J678" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K678" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L678" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M678" t="s">
+        <v>34</v>
+      </c>
+      <c r="N678" t="s">
+        <v>35</v>
+      </c>
+      <c r="O678" t="s">
+        <v>36</v>
+      </c>
+      <c r="P678" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q678" t="s">
+        <v>38</v>
+      </c>
+      <c r="R678" t="s">
+        <v>38</v>
+      </c>
+      <c r="S678" t="s">
+        <v>39</v>
+      </c>
+      <c r="V678" t="s">
+        <v>40</v>
+      </c>
+      <c r="W678" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="679" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B679" t="s">
+        <v>1410</v>
+      </c>
+      <c r="C679" t="s">
+        <v>1411</v>
+      </c>
+      <c r="D679" t="s">
+        <v>28</v>
+      </c>
+      <c r="E679" t="s">
+        <v>29</v>
+      </c>
+      <c r="F679" t="s">
+        <v>30</v>
+      </c>
+      <c r="G679" t="s">
+        <v>31</v>
+      </c>
+      <c r="H679" t="s">
+        <v>32</v>
+      </c>
+      <c r="I679" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J679" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K679" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L679" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M679" t="s">
+        <v>34</v>
+      </c>
+      <c r="N679" t="s">
+        <v>35</v>
+      </c>
+      <c r="O679" t="s">
+        <v>36</v>
+      </c>
+      <c r="P679" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q679" t="s">
+        <v>38</v>
+      </c>
+      <c r="R679" t="s">
+        <v>38</v>
+      </c>
+      <c r="S679" t="s">
+        <v>39</v>
+      </c>
+      <c r="V679" t="s">
+        <v>40</v>
+      </c>
+      <c r="W679" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="680" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B680" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C680" t="s">
+        <v>1413</v>
+      </c>
+      <c r="D680" t="s">
+        <v>28</v>
+      </c>
+      <c r="E680" t="s">
+        <v>29</v>
+      </c>
+      <c r="F680" t="s">
+        <v>30</v>
+      </c>
+      <c r="G680" t="s">
+        <v>31</v>
+      </c>
+      <c r="H680" t="s">
+        <v>32</v>
+      </c>
+      <c r="I680" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J680" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K680" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L680" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M680" t="s">
+        <v>34</v>
+      </c>
+      <c r="N680" t="s">
+        <v>35</v>
+      </c>
+      <c r="O680" t="s">
+        <v>36</v>
+      </c>
+      <c r="P680" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q680" t="s">
+        <v>38</v>
+      </c>
+      <c r="R680" t="s">
+        <v>38</v>
+      </c>
+      <c r="S680" t="s">
+        <v>39</v>
+      </c>
+      <c r="V680" t="s">
+        <v>40</v>
+      </c>
+      <c r="W680" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="681" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B681" t="s">
+        <v>1414</v>
+      </c>
+      <c r="C681" t="s">
+        <v>1415</v>
+      </c>
+      <c r="D681" t="s">
+        <v>28</v>
+      </c>
+      <c r="E681" t="s">
+        <v>29</v>
+      </c>
+      <c r="F681" t="s">
+        <v>30</v>
+      </c>
+      <c r="G681" t="s">
+        <v>31</v>
+      </c>
+      <c r="H681" t="s">
+        <v>32</v>
+      </c>
+      <c r="I681" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J681" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K681" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L681" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M681" t="s">
+        <v>34</v>
+      </c>
+      <c r="N681" t="s">
+        <v>35</v>
+      </c>
+      <c r="O681" t="s">
+        <v>36</v>
+      </c>
+      <c r="P681" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q681" t="s">
+        <v>38</v>
+      </c>
+      <c r="R681" t="s">
+        <v>38</v>
+      </c>
+      <c r="S681" t="s">
+        <v>39</v>
+      </c>
+      <c r="V681" t="s">
+        <v>40</v>
+      </c>
+      <c r="W681" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="682" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B682" t="s">
+        <v>1416</v>
+      </c>
+      <c r="C682" t="s">
+        <v>1417</v>
+      </c>
+      <c r="D682" t="s">
+        <v>28</v>
+      </c>
+      <c r="E682" t="s">
+        <v>29</v>
+      </c>
+      <c r="F682" t="s">
+        <v>30</v>
+      </c>
+      <c r="G682" t="s">
+        <v>31</v>
+      </c>
+      <c r="H682" t="s">
+        <v>32</v>
+      </c>
+      <c r="I682" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J682" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K682" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L682" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M682" t="s">
+        <v>34</v>
+      </c>
+      <c r="N682" t="s">
+        <v>35</v>
+      </c>
+      <c r="O682" t="s">
+        <v>36</v>
+      </c>
+      <c r="P682" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q682" t="s">
+        <v>38</v>
+      </c>
+      <c r="R682" t="s">
+        <v>38</v>
+      </c>
+      <c r="S682" t="s">
+        <v>39</v>
+      </c>
+      <c r="V682" t="s">
+        <v>40</v>
+      </c>
+      <c r="W682" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="683" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B683" t="s">
+        <v>1418</v>
+      </c>
+      <c r="C683" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D683" t="s">
+        <v>28</v>
+      </c>
+      <c r="E683" t="s">
+        <v>29</v>
+      </c>
+      <c r="F683" t="s">
+        <v>30</v>
+      </c>
+      <c r="G683" t="s">
+        <v>31</v>
+      </c>
+      <c r="H683" t="s">
+        <v>32</v>
+      </c>
+      <c r="I683" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J683" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K683" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L683" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M683" t="s">
+        <v>34</v>
+      </c>
+      <c r="N683" t="s">
+        <v>35</v>
+      </c>
+      <c r="O683" t="s">
+        <v>36</v>
+      </c>
+      <c r="P683" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q683" t="s">
+        <v>38</v>
+      </c>
+      <c r="R683" t="s">
+        <v>38</v>
+      </c>
+      <c r="S683" t="s">
+        <v>39</v>
+      </c>
+      <c r="V683" t="s">
+        <v>40</v>
+      </c>
+      <c r="W683" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="684" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B684" t="s">
+        <v>1420</v>
+      </c>
+      <c r="C684" t="s">
+        <v>1421</v>
+      </c>
+      <c r="D684" t="s">
+        <v>28</v>
+      </c>
+      <c r="E684" t="s">
+        <v>29</v>
+      </c>
+      <c r="F684" t="s">
+        <v>30</v>
+      </c>
+      <c r="G684" t="s">
+        <v>31</v>
+      </c>
+      <c r="H684" t="s">
+        <v>32</v>
+      </c>
+      <c r="I684" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J684" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K684" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L684" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M684" t="s">
+        <v>34</v>
+      </c>
+      <c r="N684" t="s">
+        <v>35</v>
+      </c>
+      <c r="O684" t="s">
+        <v>36</v>
+      </c>
+      <c r="P684" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q684" t="s">
+        <v>38</v>
+      </c>
+      <c r="R684" t="s">
+        <v>38</v>
+      </c>
+      <c r="S684" t="s">
+        <v>64</v>
+      </c>
+      <c r="V684" t="s">
+        <v>40</v>
+      </c>
+      <c r="W684" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="685" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B685" t="s">
+        <v>1422</v>
+      </c>
+      <c r="C685" t="s">
+        <v>1423</v>
+      </c>
+      <c r="D685" t="s">
+        <v>28</v>
+      </c>
+      <c r="E685" t="s">
+        <v>29</v>
+      </c>
+      <c r="F685" t="s">
+        <v>30</v>
+      </c>
+      <c r="G685" t="s">
+        <v>31</v>
+      </c>
+      <c r="H685" t="s">
+        <v>32</v>
+      </c>
+      <c r="I685" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J685" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K685" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L685" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M685" t="s">
+        <v>34</v>
+      </c>
+      <c r="N685" t="s">
+        <v>35</v>
+      </c>
+      <c r="O685" t="s">
+        <v>36</v>
+      </c>
+      <c r="P685" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q685" t="s">
+        <v>38</v>
+      </c>
+      <c r="R685" t="s">
+        <v>38</v>
+      </c>
+      <c r="S685" t="s">
+        <v>64</v>
+      </c>
+      <c r="V685" t="s">
+        <v>40</v>
+      </c>
+      <c r="W685" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="686" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B686" t="s">
+        <v>1424</v>
+      </c>
+      <c r="C686" t="s">
+        <v>1425</v>
+      </c>
+      <c r="D686" t="s">
+        <v>28</v>
+      </c>
+      <c r="E686" t="s">
+        <v>29</v>
+      </c>
+      <c r="F686" t="s">
+        <v>30</v>
+      </c>
+      <c r="G686" t="s">
+        <v>31</v>
+      </c>
+      <c r="H686" t="s">
+        <v>32</v>
+      </c>
+      <c r="I686" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J686" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K686" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L686" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M686" t="s">
+        <v>34</v>
+      </c>
+      <c r="N686" t="s">
+        <v>35</v>
+      </c>
+      <c r="O686" t="s">
+        <v>36</v>
+      </c>
+      <c r="P686" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q686" t="s">
+        <v>38</v>
+      </c>
+      <c r="R686" t="s">
+        <v>38</v>
+      </c>
+      <c r="S686" t="s">
+        <v>39</v>
+      </c>
+      <c r="V686" t="s">
+        <v>40</v>
+      </c>
+      <c r="W686" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="687" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B687" t="s">
+        <v>1426</v>
+      </c>
+      <c r="C687" t="s">
+        <v>1427</v>
+      </c>
+      <c r="D687" t="s">
+        <v>28</v>
+      </c>
+      <c r="E687" t="s">
+        <v>29</v>
+      </c>
+      <c r="F687" t="s">
+        <v>30</v>
+      </c>
+      <c r="G687" t="s">
+        <v>31</v>
+      </c>
+      <c r="H687" t="s">
+        <v>32</v>
+      </c>
+      <c r="I687" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J687" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K687" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L687" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M687" t="s">
+        <v>34</v>
+      </c>
+      <c r="N687" t="s">
+        <v>35</v>
+      </c>
+      <c r="O687" t="s">
+        <v>36</v>
+      </c>
+      <c r="P687" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q687" t="s">
+        <v>38</v>
+      </c>
+      <c r="R687" t="s">
+        <v>38</v>
+      </c>
+      <c r="S687" t="s">
+        <v>39</v>
+      </c>
+      <c r="V687" t="s">
+        <v>40</v>
+      </c>
+      <c r="W687" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="688" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B688" t="s">
+        <v>1428</v>
+      </c>
+      <c r="C688" t="s">
+        <v>1429</v>
+      </c>
+      <c r="D688" t="s">
+        <v>28</v>
+      </c>
+      <c r="E688" t="s">
+        <v>29</v>
+      </c>
+      <c r="F688" t="s">
+        <v>30</v>
+      </c>
+      <c r="G688" t="s">
+        <v>31</v>
+      </c>
+      <c r="H688" t="s">
+        <v>32</v>
+      </c>
+      <c r="I688" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J688" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K688" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L688" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M688" t="s">
+        <v>34</v>
+      </c>
+      <c r="N688" t="s">
+        <v>35</v>
+      </c>
+      <c r="O688" t="s">
+        <v>36</v>
+      </c>
+      <c r="P688" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q688" t="s">
+        <v>38</v>
+      </c>
+      <c r="R688" t="s">
+        <v>38</v>
+      </c>
+      <c r="S688" t="s">
+        <v>39</v>
+      </c>
+      <c r="V688" t="s">
+        <v>40</v>
+      </c>
+      <c r="W688" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="689" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B689" t="s">
+        <v>1430</v>
+      </c>
+      <c r="C689" t="s">
+        <v>1431</v>
+      </c>
+      <c r="D689" t="s">
+        <v>28</v>
+      </c>
+      <c r="E689" t="s">
+        <v>29</v>
+      </c>
+      <c r="F689" t="s">
+        <v>30</v>
+      </c>
+      <c r="G689" t="s">
+        <v>31</v>
+      </c>
+      <c r="H689" t="s">
+        <v>32</v>
+      </c>
+      <c r="I689" t="s">
+        <v>135</v>
+      </c>
+      <c r="J689" t="s">
+        <v>135</v>
+      </c>
+      <c r="K689" t="s">
+        <v>135</v>
+      </c>
+      <c r="L689" t="s">
+        <v>135</v>
+      </c>
+      <c r="M689" t="s">
+        <v>34</v>
+      </c>
+      <c r="N689" t="s">
+        <v>35</v>
+      </c>
+      <c r="O689" t="s">
+        <v>36</v>
+      </c>
+      <c r="P689" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q689" t="s">
+        <v>38</v>
+      </c>
+      <c r="R689" t="s">
+        <v>38</v>
+      </c>
+      <c r="S689" t="s">
+        <v>39</v>
+      </c>
+      <c r="V689" t="s">
+        <v>40</v>
+      </c>
+      <c r="W689" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="690" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B690" t="s">
+        <v>1432</v>
+      </c>
+      <c r="C690" t="s">
+        <v>1433</v>
+      </c>
+      <c r="D690" t="s">
+        <v>28</v>
+      </c>
+      <c r="E690" t="s">
+        <v>29</v>
+      </c>
+      <c r="F690" t="s">
+        <v>30</v>
+      </c>
+      <c r="G690" t="s">
+        <v>31</v>
+      </c>
+      <c r="H690" t="s">
+        <v>32</v>
+      </c>
+      <c r="I690" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J690" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K690" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L690" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M690" t="s">
+        <v>34</v>
+      </c>
+      <c r="N690" t="s">
+        <v>35</v>
+      </c>
+      <c r="O690" t="s">
+        <v>36</v>
+      </c>
+      <c r="P690" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q690" t="s">
+        <v>38</v>
+      </c>
+      <c r="R690" t="s">
+        <v>38</v>
+      </c>
+      <c r="S690" t="s">
+        <v>39</v>
+      </c>
+      <c r="V690" t="s">
+        <v>40</v>
+      </c>
+      <c r="W690" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="691" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B691" t="s">
+        <v>1434</v>
+      </c>
+      <c r="C691" t="s">
+        <v>1435</v>
+      </c>
+      <c r="D691" t="s">
+        <v>28</v>
+      </c>
+      <c r="E691" t="s">
+        <v>29</v>
+      </c>
+      <c r="F691" t="s">
+        <v>30</v>
+      </c>
+      <c r="G691" t="s">
+        <v>31</v>
+      </c>
+      <c r="H691" t="s">
+        <v>32</v>
+      </c>
+      <c r="I691" t="s">
+        <v>135</v>
+      </c>
+      <c r="J691" t="s">
+        <v>135</v>
+      </c>
+      <c r="K691" t="s">
+        <v>135</v>
+      </c>
+      <c r="L691" t="s">
+        <v>135</v>
+      </c>
+      <c r="M691" t="s">
+        <v>34</v>
+      </c>
+      <c r="N691" t="s">
+        <v>35</v>
+      </c>
+      <c r="O691" t="s">
+        <v>36</v>
+      </c>
+      <c r="P691" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q691" t="s">
+        <v>38</v>
+      </c>
+      <c r="R691" t="s">
+        <v>38</v>
+      </c>
+      <c r="S691" t="s">
+        <v>39</v>
+      </c>
+      <c r="V691" t="s">
+        <v>40</v>
+      </c>
+      <c r="W691" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="692" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B692" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C692" t="s">
+        <v>1437</v>
+      </c>
+      <c r="D692" t="s">
+        <v>28</v>
+      </c>
+      <c r="E692" t="s">
+        <v>29</v>
+      </c>
+      <c r="F692" t="s">
+        <v>30</v>
+      </c>
+      <c r="G692" t="s">
+        <v>31</v>
+      </c>
+      <c r="H692" t="s">
+        <v>32</v>
+      </c>
+      <c r="I692" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J692" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K692" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L692" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M692" t="s">
+        <v>34</v>
+      </c>
+      <c r="N692" t="s">
+        <v>35</v>
+      </c>
+      <c r="O692" t="s">
+        <v>36</v>
+      </c>
+      <c r="P692" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q692" t="s">
+        <v>38</v>
+      </c>
+      <c r="R692" t="s">
+        <v>38</v>
+      </c>
+      <c r="S692" t="s">
+        <v>39</v>
+      </c>
+      <c r="V692" t="s">
+        <v>40</v>
+      </c>
+      <c r="W692" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="693" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B693" t="s">
+        <v>1438</v>
+      </c>
+      <c r="C693" t="s">
+        <v>1439</v>
+      </c>
+      <c r="D693" t="s">
+        <v>28</v>
+      </c>
+      <c r="E693" t="s">
+        <v>29</v>
+      </c>
+      <c r="F693" t="s">
+        <v>30</v>
+      </c>
+      <c r="G693" t="s">
+        <v>31</v>
+      </c>
+      <c r="H693" t="s">
+        <v>32</v>
+      </c>
+      <c r="I693" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J693" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K693" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L693" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M693" t="s">
+        <v>34</v>
+      </c>
+      <c r="N693" t="s">
+        <v>35</v>
+      </c>
+      <c r="O693" t="s">
+        <v>36</v>
+      </c>
+      <c r="P693" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q693" t="s">
+        <v>38</v>
+      </c>
+      <c r="R693" t="s">
+        <v>38</v>
+      </c>
+      <c r="S693" t="s">
+        <v>39</v>
+      </c>
+      <c r="V693" t="s">
+        <v>40</v>
+      </c>
+      <c r="W693" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="694" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B694" t="s">
+        <v>1440</v>
+      </c>
+      <c r="C694" t="s">
+        <v>1441</v>
+      </c>
+      <c r="D694" t="s">
+        <v>28</v>
+      </c>
+      <c r="E694" t="s">
+        <v>29</v>
+      </c>
+      <c r="F694" t="s">
+        <v>30</v>
+      </c>
+      <c r="G694" t="s">
+        <v>31</v>
+      </c>
+      <c r="H694" t="s">
+        <v>32</v>
+      </c>
+      <c r="I694" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J694" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K694" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L694" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M694" t="s">
+        <v>34</v>
+      </c>
+      <c r="N694" t="s">
+        <v>35</v>
+      </c>
+      <c r="O694" t="s">
+        <v>36</v>
+      </c>
+      <c r="P694" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q694" t="s">
+        <v>38</v>
+      </c>
+      <c r="R694" t="s">
+        <v>38</v>
+      </c>
+      <c r="S694" t="s">
+        <v>39</v>
+      </c>
+      <c r="V694" t="s">
+        <v>40</v>
+      </c>
+      <c r="W694" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="695" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B695" t="s">
+        <v>1442</v>
+      </c>
+      <c r="C695" t="s">
+        <v>1443</v>
+      </c>
+      <c r="D695" t="s">
+        <v>28</v>
+      </c>
+      <c r="E695" t="s">
+        <v>29</v>
+      </c>
+      <c r="F695" t="s">
+        <v>30</v>
+      </c>
+      <c r="G695" t="s">
+        <v>31</v>
+      </c>
+      <c r="H695" t="s">
+        <v>32</v>
+      </c>
+      <c r="I695" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J695" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K695" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L695" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M695" t="s">
+        <v>34</v>
+      </c>
+      <c r="N695" t="s">
+        <v>35</v>
+      </c>
+      <c r="O695" t="s">
+        <v>36</v>
+      </c>
+      <c r="P695" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q695" t="s">
+        <v>38</v>
+      </c>
+      <c r="R695" t="s">
+        <v>38</v>
+      </c>
+      <c r="S695" t="s">
+        <v>39</v>
+      </c>
+      <c r="V695" t="s">
+        <v>40</v>
+      </c>
+      <c r="W695" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="696" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B696" t="s">
+        <v>1444</v>
+      </c>
+      <c r="C696" t="s">
+        <v>1445</v>
+      </c>
+      <c r="D696" t="s">
+        <v>28</v>
+      </c>
+      <c r="E696" t="s">
+        <v>29</v>
+      </c>
+      <c r="F696" t="s">
+        <v>30</v>
+      </c>
+      <c r="G696" t="s">
+        <v>31</v>
+      </c>
+      <c r="H696" t="s">
+        <v>32</v>
+      </c>
+      <c r="I696" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J696" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K696" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L696" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M696" t="s">
+        <v>34</v>
+      </c>
+      <c r="N696" t="s">
+        <v>35</v>
+      </c>
+      <c r="O696" t="s">
+        <v>36</v>
+      </c>
+      <c r="P696" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q696" t="s">
+        <v>38</v>
+      </c>
+      <c r="R696" t="s">
+        <v>38</v>
+      </c>
+      <c r="S696" t="s">
+        <v>39</v>
+      </c>
+      <c r="V696" t="s">
+        <v>40</v>
+      </c>
+      <c r="W696" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="697" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B697" t="s">
+        <v>1446</v>
+      </c>
+      <c r="C697" t="s">
+        <v>1447</v>
+      </c>
+      <c r="D697" t="s">
+        <v>28</v>
+      </c>
+      <c r="E697" t="s">
+        <v>29</v>
+      </c>
+      <c r="F697" t="s">
+        <v>30</v>
+      </c>
+      <c r="G697" t="s">
+        <v>31</v>
+      </c>
+      <c r="H697" t="s">
+        <v>32</v>
+      </c>
+      <c r="I697" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J697" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K697" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L697" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M697" t="s">
+        <v>34</v>
+      </c>
+      <c r="N697" t="s">
+        <v>35</v>
+      </c>
+      <c r="O697" t="s">
+        <v>36</v>
+      </c>
+      <c r="P697" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q697" t="s">
+        <v>38</v>
+      </c>
+      <c r="R697" t="s">
+        <v>38</v>
+      </c>
+      <c r="S697" t="s">
+        <v>39</v>
+      </c>
+      <c r="V697" t="s">
+        <v>40</v>
+      </c>
+      <c r="W697" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="698" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B698" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C698" t="s">
+        <v>1449</v>
+      </c>
+      <c r="D698" t="s">
+        <v>28</v>
+      </c>
+      <c r="E698" t="s">
+        <v>29</v>
+      </c>
+      <c r="F698" t="s">
+        <v>30</v>
+      </c>
+      <c r="G698" t="s">
+        <v>31</v>
+      </c>
+      <c r="H698" t="s">
+        <v>32</v>
+      </c>
+      <c r="I698" t="s">
+        <v>32</v>
+      </c>
+      <c r="J698" t="s">
+        <v>32</v>
+      </c>
+      <c r="K698" t="s">
+        <v>32</v>
+      </c>
+      <c r="L698" t="s">
+        <v>32</v>
+      </c>
+      <c r="M698" t="s">
+        <v>34</v>
+      </c>
+      <c r="N698" t="s">
+        <v>35</v>
+      </c>
+      <c r="O698" t="s">
+        <v>36</v>
+      </c>
+      <c r="P698" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q698" t="s">
+        <v>38</v>
+      </c>
+      <c r="R698" t="s">
+        <v>38</v>
+      </c>
+      <c r="S698" t="s">
+        <v>39</v>
+      </c>
+      <c r="V698" t="s">
+        <v>40</v>
+      </c>
+      <c r="W698" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="699" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B699" t="s">
+        <v>1450</v>
+      </c>
+      <c r="C699" t="s">
+        <v>1451</v>
+      </c>
+      <c r="D699" t="s">
+        <v>28</v>
+      </c>
+      <c r="E699" t="s">
+        <v>29</v>
+      </c>
+      <c r="F699" t="s">
+        <v>30</v>
+      </c>
+      <c r="G699" t="s">
+        <v>31</v>
+      </c>
+      <c r="H699" t="s">
+        <v>32</v>
+      </c>
+      <c r="I699" t="s">
+        <v>32</v>
+      </c>
+      <c r="J699" t="s">
+        <v>32</v>
+      </c>
+      <c r="K699" t="s">
+        <v>32</v>
+      </c>
+      <c r="L699" t="s">
+        <v>32</v>
+      </c>
+      <c r="M699" t="s">
+        <v>34</v>
+      </c>
+      <c r="N699" t="s">
+        <v>35</v>
+      </c>
+      <c r="O699" t="s">
+        <v>36</v>
+      </c>
+      <c r="P699" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q699" t="s">
+        <v>38</v>
+      </c>
+      <c r="R699" t="s">
+        <v>38</v>
+      </c>
+      <c r="S699" t="s">
+        <v>39</v>
+      </c>
+      <c r="V699" t="s">
+        <v>40</v>
+      </c>
+      <c r="W699" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="700" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B700" t="s">
+        <v>1452</v>
+      </c>
+      <c r="C700" t="s">
+        <v>1453</v>
+      </c>
+      <c r="D700" t="s">
+        <v>28</v>
+      </c>
+      <c r="E700" t="s">
+        <v>29</v>
+      </c>
+      <c r="F700" t="s">
+        <v>30</v>
+      </c>
+      <c r="G700" t="s">
+        <v>31</v>
+      </c>
+      <c r="H700" t="s">
+        <v>32</v>
+      </c>
+      <c r="I700" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J700" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K700" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L700" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M700" t="s">
+        <v>34</v>
+      </c>
+      <c r="N700" t="s">
+        <v>35</v>
+      </c>
+      <c r="O700" t="s">
+        <v>36</v>
+      </c>
+      <c r="P700" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q700" t="s">
+        <v>38</v>
+      </c>
+      <c r="R700" t="s">
+        <v>38</v>
+      </c>
+      <c r="S700" t="s">
+        <v>39</v>
+      </c>
+      <c r="V700" t="s">
+        <v>40</v>
+      </c>
+      <c r="W700" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="701" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B701" t="s">
+        <v>1454</v>
+      </c>
+      <c r="C701" t="s">
+        <v>1455</v>
+      </c>
+      <c r="D701" t="s">
+        <v>28</v>
+      </c>
+      <c r="E701" t="s">
+        <v>29</v>
+      </c>
+      <c r="F701" t="s">
+        <v>30</v>
+      </c>
+      <c r="G701" t="s">
+        <v>31</v>
+      </c>
+      <c r="H701" t="s">
+        <v>32</v>
+      </c>
+      <c r="I701" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J701" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K701" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L701" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M701" t="s">
+        <v>34</v>
+      </c>
+      <c r="N701" t="s">
+        <v>35</v>
+      </c>
+      <c r="O701" t="s">
+        <v>36</v>
+      </c>
+      <c r="P701" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q701" t="s">
+        <v>38</v>
+      </c>
+      <c r="R701" t="s">
+        <v>38</v>
+      </c>
+      <c r="S701" t="s">
+        <v>39</v>
+      </c>
+      <c r="V701" t="s">
+        <v>40</v>
+      </c>
+      <c r="W701" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="702" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B702" t="s">
+        <v>1456</v>
+      </c>
+      <c r="C702" t="s">
+        <v>1457</v>
+      </c>
+      <c r="D702" t="s">
+        <v>28</v>
+      </c>
+      <c r="E702" t="s">
+        <v>29</v>
+      </c>
+      <c r="F702" t="s">
+        <v>30</v>
+      </c>
+      <c r="G702" t="s">
+        <v>31</v>
+      </c>
+      <c r="H702" t="s">
+        <v>32</v>
+      </c>
+      <c r="I702" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J702" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K702" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L702" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M702" t="s">
+        <v>34</v>
+      </c>
+      <c r="N702" t="s">
+        <v>35</v>
+      </c>
+      <c r="O702" t="s">
+        <v>36</v>
+      </c>
+      <c r="P702" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q702" t="s">
+        <v>38</v>
+      </c>
+      <c r="R702" t="s">
+        <v>38</v>
+      </c>
+      <c r="S702" t="s">
+        <v>39</v>
+      </c>
+      <c r="V702" t="s">
+        <v>40</v>
+      </c>
+      <c r="W702" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="703" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B703" t="s">
+        <v>1458</v>
+      </c>
+      <c r="C703" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D703" t="s">
+        <v>28</v>
+      </c>
+      <c r="E703" t="s">
+        <v>29</v>
+      </c>
+      <c r="F703" t="s">
+        <v>30</v>
+      </c>
+      <c r="G703" t="s">
+        <v>31</v>
+      </c>
+      <c r="H703" t="s">
+        <v>32</v>
+      </c>
+      <c r="I703" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J703" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K703" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L703" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M703" t="s">
+        <v>34</v>
+      </c>
+      <c r="N703" t="s">
+        <v>35</v>
+      </c>
+      <c r="O703" t="s">
+        <v>36</v>
+      </c>
+      <c r="P703" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q703" t="s">
+        <v>38</v>
+      </c>
+      <c r="R703" t="s">
+        <v>38</v>
+      </c>
+      <c r="S703" t="s">
+        <v>39</v>
+      </c>
+      <c r="V703" t="s">
+        <v>40</v>
+      </c>
+      <c r="W703" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="704" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B704" t="s">
+        <v>1460</v>
+      </c>
+      <c r="C704" t="s">
+        <v>1461</v>
+      </c>
+      <c r="D704" t="s">
+        <v>28</v>
+      </c>
+      <c r="E704" t="s">
+        <v>29</v>
+      </c>
+      <c r="F704" t="s">
+        <v>30</v>
+      </c>
+      <c r="G704" t="s">
+        <v>31</v>
+      </c>
+      <c r="H704" t="s">
+        <v>32</v>
+      </c>
+      <c r="I704" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J704" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K704" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L704" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M704" t="s">
+        <v>34</v>
+      </c>
+      <c r="N704" t="s">
+        <v>35</v>
+      </c>
+      <c r="O704" t="s">
+        <v>36</v>
+      </c>
+      <c r="P704" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q704" t="s">
+        <v>38</v>
+      </c>
+      <c r="R704" t="s">
+        <v>38</v>
+      </c>
+      <c r="S704" t="s">
+        <v>39</v>
+      </c>
+      <c r="V704" t="s">
+        <v>40</v>
+      </c>
+      <c r="W704" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="705" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B705" t="s">
+        <v>1462</v>
+      </c>
+      <c r="C705" t="s">
+        <v>1463</v>
+      </c>
+      <c r="D705" t="s">
+        <v>28</v>
+      </c>
+      <c r="E705" t="s">
+        <v>29</v>
+      </c>
+      <c r="F705" t="s">
+        <v>30</v>
+      </c>
+      <c r="G705" t="s">
+        <v>31</v>
+      </c>
+      <c r="H705" t="s">
+        <v>32</v>
+      </c>
+      <c r="I705" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J705" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K705" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L705" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M705" t="s">
+        <v>34</v>
+      </c>
+      <c r="N705" t="s">
+        <v>35</v>
+      </c>
+      <c r="O705" t="s">
+        <v>36</v>
+      </c>
+      <c r="P705" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q705" t="s">
+        <v>38</v>
+      </c>
+      <c r="R705" t="s">
+        <v>38</v>
+      </c>
+      <c r="S705" t="s">
+        <v>39</v>
+      </c>
+      <c r="V705" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="706" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B706" t="s">
+        <v>1464</v>
+      </c>
+      <c r="C706" t="s">
+        <v>1465</v>
+      </c>
+      <c r="D706" t="s">
+        <v>28</v>
+      </c>
+      <c r="E706" t="s">
+        <v>29</v>
+      </c>
+      <c r="F706" t="s">
+        <v>30</v>
+      </c>
+      <c r="G706" t="s">
+        <v>31</v>
+      </c>
+      <c r="H706" t="s">
+        <v>32</v>
+      </c>
+      <c r="I706" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J706" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K706" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L706" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M706" t="s">
+        <v>34</v>
+      </c>
+      <c r="N706" t="s">
+        <v>35</v>
+      </c>
+      <c r="O706" t="s">
+        <v>36</v>
+      </c>
+      <c r="P706" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q706" t="s">
+        <v>38</v>
+      </c>
+      <c r="R706" t="s">
+        <v>38</v>
+      </c>
+      <c r="S706" t="s">
+        <v>39</v>
+      </c>
+      <c r="V706" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="707" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B707" t="s">
+        <v>1466</v>
+      </c>
+      <c r="C707" t="s">
+        <v>1467</v>
+      </c>
+      <c r="D707" t="s">
+        <v>28</v>
+      </c>
+      <c r="E707" t="s">
+        <v>29</v>
+      </c>
+      <c r="F707" t="s">
+        <v>30</v>
+      </c>
+      <c r="G707" t="s">
+        <v>31</v>
+      </c>
+      <c r="H707" t="s">
+        <v>32</v>
+      </c>
+      <c r="I707" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J707" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K707" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L707" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M707" t="s">
+        <v>34</v>
+      </c>
+      <c r="N707" t="s">
+        <v>35</v>
+      </c>
+      <c r="O707" t="s">
+        <v>36</v>
+      </c>
+      <c r="P707" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q707" t="s">
+        <v>38</v>
+      </c>
+      <c r="R707" t="s">
+        <v>38</v>
+      </c>
+      <c r="S707" t="s">
+        <v>39</v>
+      </c>
+      <c r="V707" t="s">
+        <v>40</v>
+      </c>
+      <c r="W707" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="708" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B708" t="s">
+        <v>1468</v>
+      </c>
+      <c r="C708" t="s">
+        <v>1469</v>
+      </c>
+      <c r="D708" t="s">
+        <v>28</v>
+      </c>
+      <c r="E708" t="s">
+        <v>29</v>
+      </c>
+      <c r="F708" t="s">
+        <v>30</v>
+      </c>
+      <c r="G708" t="s">
+        <v>31</v>
+      </c>
+      <c r="H708" t="s">
+        <v>32</v>
+      </c>
+      <c r="I708" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J708" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K708" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L708" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M708" t="s">
+        <v>34</v>
+      </c>
+      <c r="N708" t="s">
+        <v>35</v>
+      </c>
+      <c r="O708" t="s">
+        <v>36</v>
+      </c>
+      <c r="P708" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q708" t="s">
+        <v>38</v>
+      </c>
+      <c r="R708" t="s">
+        <v>38</v>
+      </c>
+      <c r="S708" t="s">
+        <v>39</v>
+      </c>
+      <c r="V708" t="s">
+        <v>40</v>
+      </c>
+      <c r="W708" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="709" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B709" t="s">
+        <v>1470</v>
+      </c>
+      <c r="C709" t="s">
+        <v>1471</v>
+      </c>
+      <c r="D709" t="s">
+        <v>28</v>
+      </c>
+      <c r="E709" t="s">
+        <v>29</v>
+      </c>
+      <c r="F709" t="s">
+        <v>30</v>
+      </c>
+      <c r="G709" t="s">
+        <v>31</v>
+      </c>
+      <c r="H709" t="s">
+        <v>32</v>
+      </c>
+      <c r="I709" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J709" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K709" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L709" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M709" t="s">
+        <v>34</v>
+      </c>
+      <c r="N709" t="s">
+        <v>35</v>
+      </c>
+      <c r="O709" t="s">
+        <v>36</v>
+      </c>
+      <c r="P709" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q709" t="s">
+        <v>38</v>
+      </c>
+      <c r="R709" t="s">
+        <v>38</v>
+      </c>
+      <c r="S709" t="s">
+        <v>39</v>
+      </c>
+      <c r="V709" t="s">
+        <v>40</v>
+      </c>
+      <c r="W709" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="710" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B710" t="s">
+        <v>1472</v>
+      </c>
+      <c r="C710" t="s">
+        <v>1473</v>
+      </c>
+      <c r="D710" t="s">
+        <v>28</v>
+      </c>
+      <c r="E710" t="s">
+        <v>29</v>
+      </c>
+      <c r="F710" t="s">
+        <v>30</v>
+      </c>
+      <c r="G710" t="s">
+        <v>31</v>
+      </c>
+      <c r="H710" t="s">
+        <v>32</v>
+      </c>
+      <c r="I710" t="s">
+        <v>63</v>
+      </c>
+      <c r="J710" t="s">
+        <v>63</v>
+      </c>
+      <c r="K710" t="s">
+        <v>63</v>
+      </c>
+      <c r="L710" t="s">
+        <v>63</v>
+      </c>
+      <c r="M710" t="s">
+        <v>34</v>
+      </c>
+      <c r="N710" t="s">
+        <v>35</v>
+      </c>
+      <c r="O710" t="s">
+        <v>36</v>
+      </c>
+      <c r="P710" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q710" t="s">
+        <v>38</v>
+      </c>
+      <c r="R710" t="s">
+        <v>38</v>
+      </c>
+      <c r="S710" t="s">
+        <v>39</v>
+      </c>
+      <c r="V710" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="711" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B711" t="s">
+        <v>1474</v>
+      </c>
+      <c r="C711" t="s">
+        <v>1475</v>
+      </c>
+      <c r="D711" t="s">
+        <v>28</v>
+      </c>
+      <c r="E711" t="s">
+        <v>29</v>
+      </c>
+      <c r="F711" t="s">
+        <v>30</v>
+      </c>
+      <c r="G711" t="s">
+        <v>31</v>
+      </c>
+      <c r="H711" t="s">
+        <v>32</v>
+      </c>
+      <c r="I711" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J711" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K711" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L711" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M711" t="s">
+        <v>34</v>
+      </c>
+      <c r="N711" t="s">
+        <v>35</v>
+      </c>
+      <c r="O711" t="s">
+        <v>36</v>
+      </c>
+      <c r="P711" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q711" t="s">
+        <v>38</v>
+      </c>
+      <c r="R711" t="s">
+        <v>38</v>
+      </c>
+      <c r="S711" t="s">
+        <v>39</v>
+      </c>
+      <c r="V711" t="s">
+        <v>40</v>
+      </c>
+      <c r="W711" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="712" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B712" t="s">
+        <v>1476</v>
+      </c>
+      <c r="C712" t="s">
+        <v>1477</v>
+      </c>
+      <c r="D712" t="s">
+        <v>28</v>
+      </c>
+      <c r="E712" t="s">
+        <v>29</v>
+      </c>
+      <c r="F712" t="s">
+        <v>30</v>
+      </c>
+      <c r="G712" t="s">
+        <v>31</v>
+      </c>
+      <c r="H712" t="s">
+        <v>32</v>
+      </c>
+      <c r="I712" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J712" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K712" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L712" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M712" t="s">
+        <v>34</v>
+      </c>
+      <c r="N712" t="s">
+        <v>35</v>
+      </c>
+      <c r="O712" t="s">
+        <v>36</v>
+      </c>
+      <c r="P712" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q712" t="s">
+        <v>38</v>
+      </c>
+      <c r="R712" t="s">
+        <v>38</v>
+      </c>
+      <c r="S712" t="s">
+        <v>39</v>
+      </c>
+      <c r="V712" t="s">
+        <v>40</v>
+      </c>
+      <c r="W712" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="713" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B713" t="s">
+        <v>1478</v>
+      </c>
+      <c r="C713" t="s">
+        <v>1479</v>
+      </c>
+      <c r="D713" t="s">
+        <v>28</v>
+      </c>
+      <c r="E713" t="s">
+        <v>29</v>
+      </c>
+      <c r="F713" t="s">
+        <v>30</v>
+      </c>
+      <c r="G713" t="s">
+        <v>31</v>
+      </c>
+      <c r="H713" t="s">
+        <v>32</v>
+      </c>
+      <c r="I713" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J713" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K713" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L713" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M713" t="s">
+        <v>34</v>
+      </c>
+      <c r="N713" t="s">
+        <v>35</v>
+      </c>
+      <c r="O713" t="s">
+        <v>36</v>
+      </c>
+      <c r="P713" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q713" t="s">
+        <v>38</v>
+      </c>
+      <c r="R713" t="s">
+        <v>38</v>
+      </c>
+      <c r="S713" t="s">
+        <v>39</v>
+      </c>
+      <c r="V713" t="s">
+        <v>40</v>
+      </c>
+      <c r="W713" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="714" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B714" t="s">
+        <v>1480</v>
+      </c>
+      <c r="C714" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D714" t="s">
+        <v>28</v>
+      </c>
+      <c r="E714" t="s">
+        <v>29</v>
+      </c>
+      <c r="F714" t="s">
+        <v>30</v>
+      </c>
+      <c r="G714" t="s">
+        <v>31</v>
+      </c>
+      <c r="H714" t="s">
+        <v>32</v>
+      </c>
+      <c r="I714" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J714" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K714" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L714" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M714" t="s">
+        <v>34</v>
+      </c>
+      <c r="N714" t="s">
+        <v>35</v>
+      </c>
+      <c r="O714" t="s">
+        <v>36</v>
+      </c>
+      <c r="P714" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q714" t="s">
+        <v>38</v>
+      </c>
+      <c r="R714" t="s">
+        <v>38</v>
+      </c>
+      <c r="S714" t="s">
+        <v>39</v>
+      </c>
+      <c r="V714" t="s">
+        <v>40</v>
+      </c>
+      <c r="W714" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="715" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B715" t="s">
+        <v>1482</v>
+      </c>
+      <c r="C715" t="s">
+        <v>1483</v>
+      </c>
+      <c r="D715" t="s">
+        <v>28</v>
+      </c>
+      <c r="E715" t="s">
+        <v>29</v>
+      </c>
+      <c r="F715" t="s">
+        <v>30</v>
+      </c>
+      <c r="G715" t="s">
+        <v>31</v>
+      </c>
+      <c r="H715" t="s">
+        <v>32</v>
+      </c>
+      <c r="I715" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J715" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K715" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L715" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M715" t="s">
+        <v>34</v>
+      </c>
+      <c r="N715" t="s">
+        <v>35</v>
+      </c>
+      <c r="O715" t="s">
+        <v>36</v>
+      </c>
+      <c r="P715" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q715" t="s">
+        <v>38</v>
+      </c>
+      <c r="R715" t="s">
+        <v>38</v>
+      </c>
+      <c r="S715" t="s">
+        <v>39</v>
+      </c>
+      <c r="V715" t="s">
+        <v>40</v>
+      </c>
+      <c r="W715" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="716" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B716" t="s">
+        <v>1484</v>
+      </c>
+      <c r="C716" t="s">
+        <v>1485</v>
+      </c>
+      <c r="D716" t="s">
+        <v>28</v>
+      </c>
+      <c r="E716" t="s">
+        <v>29</v>
+      </c>
+      <c r="F716" t="s">
+        <v>30</v>
+      </c>
+      <c r="G716" t="s">
+        <v>31</v>
+      </c>
+      <c r="H716" t="s">
+        <v>32</v>
+      </c>
+      <c r="I716" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J716" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K716" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L716" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M716" t="s">
+        <v>34</v>
+      </c>
+      <c r="N716" t="s">
+        <v>35</v>
+      </c>
+      <c r="O716" t="s">
+        <v>36</v>
+      </c>
+      <c r="P716" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q716" t="s">
+        <v>38</v>
+      </c>
+      <c r="R716" t="s">
+        <v>38</v>
+      </c>
+      <c r="S716" t="s">
+        <v>39</v>
+      </c>
+      <c r="V716" t="s">
+        <v>40</v>
+      </c>
+      <c r="W716" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="717" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B717" t="s">
+        <v>1486</v>
+      </c>
+      <c r="C717" t="s">
+        <v>1487</v>
+      </c>
+      <c r="D717" t="s">
+        <v>28</v>
+      </c>
+      <c r="E717" t="s">
+        <v>29</v>
+      </c>
+      <c r="F717" t="s">
+        <v>30</v>
+      </c>
+      <c r="G717" t="s">
+        <v>31</v>
+      </c>
+      <c r="H717" t="s">
+        <v>32</v>
+      </c>
+      <c r="I717" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J717" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K717" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L717" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M717" t="s">
+        <v>34</v>
+      </c>
+      <c r="N717" t="s">
+        <v>35</v>
+      </c>
+      <c r="O717" t="s">
+        <v>36</v>
+      </c>
+      <c r="P717" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q717" t="s">
+        <v>38</v>
+      </c>
+      <c r="R717" t="s">
+        <v>38</v>
+      </c>
+      <c r="S717" t="s">
+        <v>39</v>
+      </c>
+      <c r="V717" t="s">
+        <v>40</v>
+      </c>
+      <c r="W717" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="718" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B718" t="s">
+        <v>1488</v>
+      </c>
+      <c r="C718" t="s">
+        <v>1489</v>
+      </c>
+      <c r="D718" t="s">
+        <v>28</v>
+      </c>
+      <c r="E718" t="s">
+        <v>29</v>
+      </c>
+      <c r="F718" t="s">
+        <v>30</v>
+      </c>
+      <c r="G718" t="s">
+        <v>31</v>
+      </c>
+      <c r="H718" t="s">
+        <v>32</v>
+      </c>
+      <c r="I718" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J718" t="s">
+        <v>1397</v>
+      </c>
+      <c r="K718" t="s">
+        <v>1397</v>
+      </c>
+      <c r="L718" t="s">
+        <v>1397</v>
+      </c>
+      <c r="M718" t="s">
+        <v>34</v>
+      </c>
+      <c r="N718" t="s">
+        <v>35</v>
+      </c>
+      <c r="O718" t="s">
+        <v>36</v>
+      </c>
+      <c r="P718" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q718" t="s">
+        <v>38</v>
+      </c>
+      <c r="R718" t="s">
+        <v>38</v>
+      </c>
+      <c r="S718" t="s">
+        <v>39</v>
+      </c>
+      <c r="V718" t="s">
+        <v>40</v>
+      </c>
+      <c r="W718" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>